<commit_message>
Add AI Audit Log - SWD392 Week2
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamHongQuan.xlsx
+++ b/AI Audit Log_PhamHongQuan.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Template" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Week1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Week2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -690,4 +691,203 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="95" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Giai đoạn/Thành phần DTC</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Nội dung Prompt (Câu lệnh)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Phản hồi của AI &amp; Quyết định của người học (Reflection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Decomposition – Phân rã hệ thống thành các use case</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>"Hệ thống IELTSPhobic có 4 actor: Guest (chưa đăng nhập), Learner (học viên), Moderator (quản lý forum), Admin. Hệ thống có các chức năng chính: thi Reading/Listening/Writing/Speaking, từ điển, diễn đàn, VIP, quản lý người dùng. Làm sao tôi phân rã và xác định các use case cho từng actor?"</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý chia use case theo actor: mỗi actor có một use case diagram riêng. AI liệt kê sơ bộ: Guest → Register, Login; Learner → Take Exam, View Result, Use Dictionary, Post Forum, Upgrade VIP; Moderator → Manage Posts, Manage Comments; Admin → Manage Users, Manage Exams, Manage VipPlans.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: Cách chia riêng từng actor của AI dễ hiểu nhưng không thể hiện được mối quan hệ giữa các use case. Một số use case xuất hiện ở nhiều actor (vd: View Profile có ở Learner, Moderator, Admin) – nếu vẽ riêng sẽ bị trùng lặp.
+• Contextualization: AI không biết rằng IELTSPhobic có sự phân cấp role: Moderator kế thừa quyền của Learner (vẫn thi được), Admin cũng có thể làm Moderator. Cần thể hiện generalization giữa các actor.
+• Creative Synthesis: Tôi thiết kế use case diagram với actor hierarchy: User (general) → Learner (thi, từ điển) → Moderator (quản lý nội dung) → Admin (quản trị hệ thống). Use case "Take Exam" được chia nhỏ: "Take Reading Test", "Take Listening Test", "Take Writing Test", "Take Speaking Test" – dùng &lt;&lt;include&gt;&gt; cho các hành vi chung như "Submit Answer", "View Result".
+• Decision Ownership: Quyết định vẽ một use case diagram tổng thể với actor generalization thay vì tách riêng. Lý do: thể hiện đúng quan hệ giữa các actor, tránh trùng lặp use case.
+EVIDENCE: Use case diagram – các use case Take Reading/Listening/Writing/Speaking Test gắn với "exam page navigation" và "Listening exam page" commits (Oct 9, 22).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Phân biệt Include và Extend trong use case</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>"Trong use case diagram IELTSPhobic, "Submit Exam" luôn kéo theo "Grade Exam" và "Save Attempt". Tôi nên dùng &lt;&lt;include&gt;&gt; hay &lt;&lt;extend&gt;&gt;? Và "View Result" chỉ xảy ra sau khi nộp bài – đó là quan hệ gì?"</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI trả lời "cả hai đều dùng &lt;&lt;extend&gt;&gt; vì đều xảy ra sau khi nộp bài". AI giải thích extend là "hành vi mở rộng, xảy ra sau hành vi chính".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Logic Error]: AI hoàn toàn sai. &lt;&lt;extend&gt;&gt; dùng cho hành vi TÙY CHỌN (optional behavior), không phải hành vi xảy ra "sau". "Grade Exam" và "Save Attempt" là bắt buộc mỗi khi nộp bài – phải dùng &lt;&lt;include&gt;&gt;. "View Result" cũng là bắt buộc sau khi nộp (hoặc có thể xem sau) nhưng là một use case riêng, liên kết bằng association bình thường, không phải include hay extend.
+• Contextualization: AI không hiểu rõ business rule: "Grade Exam" và "Save Attempt" luôn chạy ngầm khi submit – người dùng không tương tác trực tiếp. Đây chính là tình huống kinh điển của &lt;&lt;include&gt;&gt;.
+• Creative Synthesis: Tôi sửa: "Take Reading Test" &lt;&lt;include&gt;&gt; "Submit Answer" và "Submit Answer" &lt;&lt;include&gt;&gt; "Grade Test" + "Save Attempt". "View Result" là use case riêng, không dùng include/extend với Submit.
+• Decision Ownership: Quyết định đúng quan hệ &lt;&lt;include&gt;&gt; cho các hành vi bắt buộc, không dùng &lt;&lt;extend&gt;&gt; tùy tiện như AI. Lý do: đúng chuẩn UML, thể hiện đúng business rule.
+CORRECTIVE ACTION: Sửa use case diagram – đổi quan hệ sai từ &lt;&lt;extend&gt;&gt; sang &lt;&lt;include&gt;&gt;.
+EVIDENCE: Class diagram và sequence diagram sau này phản ánh đúng luồng Submit → Grade → Save.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Pattern Recognition – Xác định Primary và Secondary Actor</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>"Trong use case "Upgrade to VIP", ngoài Learner ra còn có Stripe Payment Gateway. Stripe có phải actor không? Nếu có thì là primary hay secondary? Còn OpenAI – khi user "Get Writing Feedback" thì AI có phải là actor?"</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI trả lời Stripe và OpenAI không phải actor vì "chúng là hệ thống, không phải người dùng". AI nói chỉ con người mới là actor.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION]: AI sai. Trong UML, actor KHÔNG chỉ là con người – actor là bất kỳ thực thể nào tương tác với hệ thống, bao gồm cả hệ thống ngoài (external systems). Stripe và OpenAI là secondary actor (hỗ trợ, không khởi tạo use case).
+• Contextualization: AI không biết rằng trong mô hình của IELTSPhobic: Stripe xử lý thanh toán, OpenAI chấm bài Writing/Speaking, Cloudinary lưu file. Đây đều là external systems – cần được mô hình hóa rõ ràng.
+• Creative Synthesis: Tôi xác định: Learner là primary actor (khởi tạo use case "Upgrade to VIP"), Stripe là secondary actor (hỗ trợ use case). Tương tự: Learner → "Get Writing Feedback" (primary), OpenAI → trả lời (secondary). Thêm stereotype «external system» để phân biệt.
+• Decision Ownership: Quyết định đưa Stripe, OpenAI, Cloudinary vào use case diagram với vai trò secondary actor. Lý do: mô hình hóa đúng UML, thể hiện đầy đủ các thành phần tương tác.
+EVIDENCE: External services trong project: stripe payment, OpenAIService, CloudinaryService.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Abstraction – Các loại quan hệ giữa các Use Case</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>"Theo tôi tìm hiểu, UML có 4 loại quan hệ use case: Association, Generalization, Include, Extend. Nhưng tôi thấy một số tài liệu còn có Import và Access. Tôi nên dùng những quan hệ nào cho IELTSPhobic?"</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI liệt kê 4 quan hệ: Association, Generalization, &lt;&lt;include&gt;&gt;, &lt;&lt;extend&gt;&gt;. AI nói Import và Access "không phải UML chuẩn, có thể bỏ qua".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI lần này ĐÚNG về 4 quan hệ chính nhưng thiếu chính xác về nguồn gốc. Import và Access thực ra là từ ngữ cảnh khác (Access trong use case của UP, Import trong UML 1.x) – đúng là không cần dùng.
+• Contextualization: Trong IELTSPhobic, 4 quan hệ cơ bản đã đủ: (1) Association kết nối actor với use case, (2) Generalization cho actor hierarchy, (3) &lt;&lt;include&gt;&gt; cho "Submit Answer" → "Grade Test", (4) &lt;&lt;extend&gt;&gt; cho các hành vi tùy chọn (vd: "View Dictionary" extend "Take Reading Test" – từ điển nổi, không bắt buộc).
+• Creative Synthesis: Tôi xác nhận lại với UML 2.5.1 spec – chỉ 4 quan hệ là chuẩn. Áp dụng cho IELTSPhobic: Association (nối actor-use case), Generalization (User→Learner→Moderator→Admin), &lt;&lt;include&gt;&gt; (bắt buộc), &lt;&lt;extend&gt;&gt; (tùy chọn).
+• Decision Ownership: Giữ 4 quan hệ như AI liệt kê. Thêm ghi chú: &lt;&lt;extend&gt;&gt; chỉ dùng cho hành vi thực sự optional (vd: dictionary popup trong khi thi). Lý do: không làm phức tạp diagram.
+EVIDENCE: Use case diagram IELTSPhobic với 4 loại quan hệ được đánh dấu rõ ràng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Algorithms – Mô hình hóa luồng nghiệp vụ "Take Exam"</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>"Tôi cần mô hình hóa use case "Take Reading Test" từ lúc user mở đề đến lúc xem kết quả. Nên dùng activity diagram hay use case description để mô tả?"</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI khuyên dùng cả hai: use case description cho văn bản, activity diagram cho hình ảnh. AI gợi ý activity diagram tuyến tính: Start → Show Passage → Show Questions → User Answers → Submit → Grade → Show Result.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: Activity diagram AI đề xuất quá tuyến tính và bỏ qua các rẽ nhánh quan trọng: (1) Timer hết → tự động nộp (forced submit), (2) User chưa trả lời hết → confirm nộp, (3) Lưu nháp tạm thời (auto-save).
+• Contextualization: AI không biết IELTSPhobic có chức năng auto-save answers mỗi 30 giây, và forced submit khi hết giờ. Đây là business rules quan trọng.
+• Creative Synthesis: Tôi thiết kế activity diagram với: (1) Timer check song song với answering, (2) Decision node "hết giờ?" → forced submit, (3) Decision node "đã trả lời hết?" → confirm dialog, (4) Parallel: vừa grade vừa lưu attempt.
+• Decision Ownership: Quyết định vẽ activity diagram không tuyến tính, có các fork/join cho timer song song. Lý do: phản ánh đúng luồng thực tế, không oversimplify.
+EVIDENCE: Component ExamRenderer với useExamTimer hook; commit "change submission structure" (Oct 27, 963ac39) thể hiện luồng submit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Abstraction – Xác định phạm vi hệ thống (System Boundary)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>"IELTSPhobic tương tác với nhiều hệ thống ngoài: OpenAI (chấm bài), Stripe (thanh toán), Cloudinary (lưu file), Firebase Auth (xác thực). Những hệ thống này có nằm trong system boundary của IELTSPhobic không? Vẽ thế nào?"</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI nói tất cả hệ thống ngoài đều nằm NGOÀI system boundary, chỉ vẽ một box duy nhất cho IELTSPhobic. AI bảo "không cần vẽ chi tiết".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI đúng về việc external systems nằm ngoài system boundary. Tuy nhiên, trong use case diagram, không chỉ vẽ 1 box đơn giản – cần vẽ rõ IELTSPhobic (bên trong box) và các actor/system bên ngoài. AI oversimplify bằng cách không phân biệt primary/secondary actor.
+• Contextualization: AI không biết rằng UML cho phép vẽ external systems như actor với stereotype «external system». Việc này giúp người đọc hiểu ngay hệ thống phụ thuộc vào những gì.
+• Creative Synthesis: Tôi vẽ: system boundary box "IELTSPhobic" chứa tất cả use case. Bên ngoài box: Learner (primary), Stripe (secondary, «external system»), OpenAI (secondary), Cloudinary (secondary). Mỗi external system chỉ kết nối với use case liên quan.
+• Decision Ownership: Quyết định vẽ system boundary rõ ràng với primary actor bên trái và secondary actor bên phải (phân biệt bằng stereotype). Lý do: dễ đọc, thể hiện đúng kiến trúc tổng thể.
+EVIDENCE: Các external services trong project: IOpenAIService.cs, ICloudinaryService.cs, StripePaymentService.cs; biểu diễn trong use case diagram.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add AI Audit Log - SWD392 Week3
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamHongQuan.xlsx
+++ b/AI Audit Log_PhamHongQuan.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Template" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Week1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Week2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Week3" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -890,4 +891,221 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="95" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Giai đoạn/Thành phần DTC</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Nội dung Prompt (Câu lệnh)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Phản hồi của AI &amp; Quyết định của người học (Reflection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Abstraction – Xác định Entity Classes từ yêu cầu hệ thống</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>"Theo phương pháp Static Modeling (Ch07), hãy xác định các entity classes chính của IELTSPhobic từ đặc tả use case. Có nên tạo class cho mọi danh từ xuất hiện trong use case description không?"</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý dùng kỹ thuật "noun extraction" – gạch chân tất cả danh từ rồi biến mỗi danh từ thành một class. AI liệt kê ~30 class: User, Exam, Question, Answer, Score, Forum, Post, Comment, Dictionary, Word, Plan, Payment, Button, Page, Screen...
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [OVERSIMPLIFICATION]: Gợi ý "mỗi danh từ một class" của AI quá máy móc. Button, Page, Screen là UI elements – không phải entity class. Email cũng là service, không phải thực thể lưu trữ. Entity class là thứ có TRẠNG THÁI cần lưu trữ lâu dài.
+• Contextualization: AI không biết rằng trong database của IELTSPhobic, chỉ có các bảng cụ thể: User, Exam, Reading, Listening, Speaking, Writing, Question, Attempt, Post, Comment, Transaction, VipPlan.
+• Creative Synthesis: Tôi phân loại theo 3 stereotype của Gomaa: 
+  - Entity class (lưu trạng thái): User, Exam, Reading, Listening, Writing, Speaking, Question, ExamAttempt, Post, Comment, VipPlan, Transaction, VocabGroup, Word, Notification, Report
+  - Boundary class (giao tiếp ngoài): OpenAIService, StripeGateway, CloudinaryService
+  - Control class (điều phối): ExamController, AuthController, PostController, PaymentController...
+• Decision Ownership: Quyết định giữ 16 entity classes cốt lõi, loại ~14 danh từ rác (Button, Page, Screen...). Lý do: class diagram phải phản ánh đúng các bảng dữ liệu thật.
+EVIDENCE: Các Model file trong WebAPI/Models/ (User.cs, Exam.cs, Reading.cs, Listening.cs...); commit "back end for reading and listening" (Oct 27, 0fac605).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Phân biệt Composition và Aggregation</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>"Trong IELTSPhobic, Test gồm nhiều Question, và Question thuộc về Test. Còn Learner tạo nhiều ForumPost. Quan hệ nào là Composition? Quan hệ nào là Aggregation?"</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI trả lời CẢ HAI đều là Composition (hình thoi đặc) vì "đều là has-a mạnh, một cái chứa cái kia".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Logic Error]: AI sai. Composition hàm ý vòng đời PHỤ THUỘC – khi đối tượng chứa bị xóa, đối tượng con cũng bị xóa. Aggregation là whole-part lỏng, con tồn tại độc lập.
+  - Test – Question: Composition (xóa Test thì Question đi theo, vì Question không tồn tại nếu không có Test)
+  - User – ForumPost: Association (xóa User, các bài post forum vẫn được lưu "[deleted user]" – post sống độc lập)
+• Contextualization: AI không biết business rule: IELTSPhobic giữ lại bài viết cả khi user xóa tài khoản để bảo toàn ngữ cảnh diễn đàn.
+• Creative Synthesis: Test ◆— Question là Composition (cascade delete). Learner —— ForumPost là Association 1-nhiều (không cascade). Thêm multiplicity rõ ràng.
+• Decision Ownership: Đúng loại quan hệ. Lý do: chọn sai sẽ kéo theo thiết kế khóa ngoại cascade delete sai trong DB.
+CORRECTIVE ACTION: Sửa class diagram – đổi User→ForumPost từ Composition sang Association.
+EVIDENCE: Database schema với ràng buộc khóa ngoại; Model Comment.cs và Post.cs có ForeignKey attributes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Abstraction – Mô hình hóa Test Attempt và quan hệ nhiều-nhiều</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>"Trong IELTSPhobic, một User có thể làm nhiều Exam, và một Exam có thể được làm bởi nhiều User. Đây là quan hệ many-to-many. Làm sao mô hình hóa điều này trong class diagram?"</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý dùng Association Class tên ExamAttempt giữa User và Exam. AI giải thích: ExamAttempt lưu thông tin thêm như attemptId, score, startTime, endTime.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [ĐÚNG]: Lần này AI ĐÚNG. Association Class là cách chuẩn để xử lý many-to-many kèm thuộc tính. Tôi kiểm chứng bằng Ch07: Association Class được dùng khi quan hệ có dữ liệu riêng.
+• Contextualization: AI không biết chi tiết: một Exam có thể có nhiều Attempt của cùng một User (user làm đi làm lại). Đây là unary many-to-many hay self-referencing không phải – đơn giản là User và Exam có quan hệ 1-nhiều qua Attempt.
+• Creative Synthesis: Tôi thiết kế: User 1 — 0..* ExamAttempt, Exam 1 — 0..* ExamAttempt. ExamAttempt có: attemptId, userId, examId, startTime, endTime, rawScore, bandScore, status (InProgress/Submitted/Graded), answers (danh sách AnswerAttempt).
+• Decision Ownership: Giữ Association Class như AI đề xuất nhưng mở rộng: thêm status và answers chi tiết. Lý do: phản ánh đúng nhu cầu lưu nhiều attempt, có tracking trạng thái.
+EVIDENCE: Model ExamAttempt.cs; commit "change submission structure" (Oct 27, 963ac39).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Abstraction – UML Stereotype và phân loại Boundary/Control/Entity</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>"Theo COMET (Ch07), class được phân loại bằng stereotype «entity», «boundary», «control». Trong IELTSPhobic, OpenAIService gọi API chấm bài – đó là boundary hay control class? Còn ExamController?"</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI trả lời OpenAIService là boundary (vì giao tiếp hệ thống ngoài), ExamController là control. AI giải thích đúng theo mô hình BCE.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI ĐÚNG. Boundary class là cầu nối giữa hệ thống và actor/hệ thống ngoài; control class điều phối luồng; entity class lưu trạng thái.
+• Contextualization: AI không phân biệt một sắc thái: trong code thực tế, OpenAIService vừa làm boundary (gọi HTTP) vừa chứa logic ghép prompt – dễ bị lẫn vai trò.
+• Creative Synthesis: Tôi tách: OpenAIClient là boundary thuần (chỉ gửi/nhận HTTP), FeedbackController là control (kiểm tra VIP, ghép prompt, gọi client, lưu kết quả), Feedback là entity (lưu nội dung feedback).
+• Decision Ownership: Mỗi class một stereotype, tuân thủ SRP. Lý do: tránh lẫn trách nhiệm, dễ test.
+EVIDENCE: Các service: IOpenAIService.cs, ISpeechToTextService.cs, StripeWebhookService.cs được phân tầng BCE trong class diagram.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Decomposition – Generalization hierarchy cho User và Exam</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>"IELTSPhobic có 3 loại user: Learner, Moderator, Admin. Còn Exam có 4 loại: Reading, Listening, Writing, Speaking. Mô hình hóa bằng generalization thế nào?"</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI đề xuất: class User (base) → 3 class con; class Exam (base) → 4 class con. AI không đề cập abstract class hay method trừu tượng.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI đúng về hướng generalization nhưng thiếu chi tiết quan trọng. Theo Ch07: nếu class cha không bao giờ được instantiate trực tiếp, phải đánh dấu abstract (in nghiêng tên class). User và Exam đều là abstract.
+• Contextualization: AI không nắm được rằng method gradeTest() có implementation khác nhau cho từng loại exam – cần thể hiện polymorphism.
+• Creative Synthesis: Tôi thiết kế:
+  - «abstract» User {+userId, +email, +role} ← Learner, Moderator, Admin
+  - «abstract» Exam {+examId, +title, +duration; +abstract gradeTest()} ← Reading, Listening, Writing, Speaking
+  - Reading và Listening override gradeTest() (auto-graded), Writing và Speaking override với AI feedback.
+• Decision Ownership: Dùng cây thừa kế 2 tầng với abstract class. Lý do: thể hiện đúng is-a relationship, dùng polymorphism cho gradeTest().
+EVIDENCE: Các Model: User.cs (base), không có class Learner/Moderator/Admin riêng (dùng role enum) – thể hiện sự khác biệt giữa lý thuyết và thực tế implement. Exam là abstract, gradeTest() implement ở Service layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Pattern Recognition – Xác định multiplicity và constraints</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>"Trong class diagram, một Reading có nhiều Question. Một User có thể có 0 hoặc nhiều Transaction. Làm sao xác định và biểu diễn multiplicity chính xác?"</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý multiplicity mặc định: 1 — 0..* cho hầu hết quan hệ. AI nói "không cần quá chi tiết, 1 — * là đủ".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [OVERSIMPLIFICATION]: Multiplicity phải chính xác, không thể "mặc định". Sai multiplicity sẽ dẫn đến sai ràng buộc DB và sai logic nghiệp vụ.
+  - Exam 1 —— 1..* Question (một exam phải có ít nhất 1 câu hỏi)
+  - User 1 —— 0..* ExamAttempt (user có thể chưa làm bài nào)
+  - Exam 1 —— 0..* ExamAttempt (exam có thể chưa ai làm)
+  - Learner 1 —— 0..* VipTransaction (có thể chưa mua VIP)
+• Contextualization: AI không biết business rule cụ thể của từng cặp class.
+• Creative Synthesis: Tôi xác định multiplicity cho từng quan hệ dựa trên business rules:
+  - Exam 1 — 1..* Question (bắt buộc có câu hỏi)
+  - Question 1 — 1..* Answer (mỗi câu hỏi có ít nhất 1 đáp án)
+  - User 1 — 0..* Post (có thể chưa post)
+  - Post 1 — 0..1..* Attachment (có thể không có file đính kèm)
+  - Post 1 — 0..* Comment
+  - User 1 — 0..1 VipPlan (có thể chưa có VIP)
+• Decision Ownership: Multiplicity chính xác cho mọi quan hệ. Lý do: đảm bảo class diagram khớp với database schema thực tế.
+EVIDENCE: Database schema với các ràng buộc NOT NULL, Foreign Key; Model files với [Required] attributes.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add AI Audit Log - SWD392 Week4
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamHongQuan.xlsx
+++ b/AI Audit Log_PhamHongQuan.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Week1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Week2" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Week3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Week4" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1108,4 +1109,228 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="95" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Giai đoạn/Thành phần DTC</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Nội dung Prompt (Câu lệnh)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Phản hồi của AI &amp; Quyết định của người học (Reflection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Decomposition – Phân tầng lifeline cho Sequence Diagram</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>"Tôi vẽ sequence diagram cho use case "Take Reading Test" – luồng từ lúc user mở đề đến lúc nộp bài và xem kết quả. Nên có những lifeline nào? Theo mô hình 3-layer (UI → Controller → Service → Repository)?"</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý 4 lifeline: UI, ExamController, ExamService, Database. AI nói "không cần Repository riêng, gộp vào Service cho đơn giản".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: Gộp Service và Repository của AI vi phạm nguyên tắc layered architecture. Repository layer có trách nhiệm riêng (truy xuất dữ liệu), tách biệt khỏi business logic trong Service.
+• Contextualization: AI không biết IELTSPhobic có hẳn tầng Repository riêng (UserRepository, ExamRepository, ReadingRepository...) và dùng Dependency Injection để inject vào Service.
+• Creative Synthesis: Tôi thiết kế 6 lifeline: (1) Learner (actor), (2) ReadingExamPage (UI), (3) ExamController, (4) ExamService, (5) ExamRepository, (6) Database (SQL Server). Mỗi lifeline tương ứng một tầng kiến trúc.
+• Decision Ownership: Giữ 6 lifeline, không gộp Repository vào Service. Lý do: phản ánh đúng kiến trúc thực tế, tuân thủ separation of concerns.
+EVIDENCE: Cấu trúc project WebAPI/ với Controllers/, Services/, Repositories/; commit "Exam backend" (Oct 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Combined Fragment cho luồng rẽ nhánh</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>"Trong sequence diagram "Take Reading Test", cần mô hình hóa: nếu hết giờ thì tự động nộp (forced submit), nếu chưa hết giờ thì user có thể nộp hoặc tiếp tục. Dùng combined fragment nào cho phù hợp?"</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI trả lời "dùng alt fragment cho tất cả điều kiện". AI nói alt dùng để rẽ nhánh, mỗi nhánh là một operand.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI đúng khi nói dùng alt fragment, nhưng thiếu: cần kết hợp opt fragment cho forced submit (timer) và alt cho user decision.
+  - opt fragment: "timer expires" → forced submit (optional, chỉ xảy ra nếu hết giờ)
+  - alt fragment: "user clicks submit" vs "user continues" rẽ nhánh
+• Contextualization: AI không biết IELTSPhobic có useExamTimer chạy song song, khi hết giờ tự động gọi submit API.
+• Creative Synthesis: Tôi thiết kế: (1) opt fragment [timer expired] → system tự động submit, (2) alt fragment [user action] → submit hay cancel, (3) Trong cả 2 trường hợp, sau submit là đoạn code chung (dùng ref fragment để tái sử dụng).
+• Decision Ownership: Kết hợp opt + alt + ref fragments. Lý do: chính xác với UML, thể hiện đủ các tình huống.
+EVIDENCE: useExamTimer.js hook chạy song song với component; commit "change submission structure" (Oct 27).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Algorithms – Synchronous vs Asynchronous messages</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>"Trong sequence diagram use case "Get AI Writing Feedback", UI gọi API, API gọi OpenAI – đây là synchronous hay asynchronous messages? Stripe payment callback thì sao?"</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI trả lời "tất cả đều là synchronous messages, vì HTTP là request-response". AI nói không có asynchronous trong web application.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Oversimplification]: AI sai. Stripe payment là asynchronous: user redirect sang Stripe, Stripe gọi webhook callback. Cũng có thể dùng async/await trong C# cho I/O operations – đây là asynchronous message ở mức code.
+• Contextualization: AI không biết IELTSPhobic có StripeWebhookController nhận callback từ Stripe, và OpenAI call là async I/O.
+• Creative Synthesis: Tôi phân loại:
+  - Synchronous (mũi tên đặc): UI → Controller, Controller → Service (trong cùng system)
+  - Asynchronous (mũi tên nửa): Service → OpenAI (HTTP call async), Stripe → Webhook (callback)
+  - Return message (mũi tên đứt): trả về kết quả từ các tầng
+• Decision Ownership: Phân biệt sync/async messages đúng UML. Lý do: thể hiện chính xác bản chất tương tác, Stripe webhook là async bắt buộc phải dùng ký hiệu đúng.
+EVIDENCE: StripeWebhookController.cs nhận POST từ Stripe; OpenAIService.cs dùng HttpClient async.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Abstraction – Ký hiệu chuẩn của Sequence Diagram</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>"Theo UML, sequence diagram có những thành phần bắt buộc nào? Tôi đọc có người dùng "self-message", "creation message", "lost message" – những thứ này có cần trong diagram IELTSPhobic không?"</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI liệt kê thành phần bắt buộc: lifeline, activation bar, message, combined fragment. AI nói "self-message, lost message không cần dùng".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI đúng về thành phần cơ bản nhưng sai khi nói self-message "không cần". Self-message dùng khi object gọi method của chính nó (vd: Service tự gọi internal validation method).
+• Contextualization: Trong IELTSPhobic: ExamService.SubmitExam() → self-message ValidateSubmission() → trước khi gọi Repository. Self-message thể hiện rõ nội bộ xử lý.
+• Creative Synthesis: Tôi sử dụng:
+  - Lifeline: hình chữ nhật với tên class (vd: :ExamController)
+  - Activation bar: thanh dọc khi method active
+  - Message: mũi tên đồng bộ (→), async (→&gt;), return (- - -&gt;)
+  - Self-message: vòng cung (ExamService tự gọi internal validate)
+  - Combined fragments: alt, opt, ref
+  - Creation message: tạo object mới (vd: tạo ExamAttempt mới)
+• Decision Ownership: Bao gồm self-message, creation message trong diagram. Lý do: thể hiện đầy đủ tương tác nội bộ.
+EVIDENCE: Sequence diagram "Take Reading Test" với đầy đủ ký hiệu UML.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Algorithms – Ánh xạ message từ Sequence Diagram vào code thực tế</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>"Tôi muốn sequence diagram cho use case "Add Listening Test" (Admin thêm đề thi Listening). Các message trên diagram ánh xạ thế nào vào code ASP.NET Core thực tế?"</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI đề xuất luồng: AdminUI → ListeningController → ListeningService → ListeningRepository → DB. AI mô tả message chung chung.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI đúng về luồng cơ bản nhưng thiếu chi tiết: cần show validation (file audio, định dạng), upload file lên Cloudinary, và transaction rollback nếu lỗi.
+• Contextualization: AI không biết Listening có audio file cần upload lên Cloudinary trước, rồi mới lưu URL vào DB.
+• Creative Synthesis: Tôi vẽ sequence diagram:
+  1. Admin → AdminUI: điền form + chọn file audio
+  2. AdminUI → ListeningController: POST /api/listening (FormData)
+  3. ListeningController → ListeningService: CreateListeningAsync(dto)
+  4. ListeningService → CloudinaryService: UploadAudioAsync(file)
+  5. CloudinaryService →&gt; Cloudinary: HTTP upload (async)
+  6. Cloudinary --&gt;&gt; CloudinaryService: audioUrl
+  7. ListeningService → ListeningRepository: AddListeningAsync(data)
+  8. ListeningRepository → DB: INSERT
+  9. DB --&gt; ListeningRepository: success
+  10. (return messages tương ứng)
+• Decision Ownership: Vẽ sequence diagram chi tiết với Cloudinary upload và DB transaction. Lý do: thể hiện đúng luồng thực tế, bao gồm cả external service.
+EVIDENCE: Commit "feat(admin): enhance audio upload validation and error handling in AddListening" (Oct 31, bd7cf5c); AddListening.jsx component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Abstraction – Mức độ chi tiết: Analysis vs Design Level</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>"Khi vẽ sequence diagram cho báo cáo SWD392, tôi nên vẽ ở mức analysis (khái niệm) hay design (chi tiết với method signatures)? Mức nào phù hợp?"</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI giải thích analysis-level chỉ show tương tác khái niệm giữa các object, design-level show method signatures cụ thể. AI khuyên dùng analysis-level vì "dễ vẽ và dễ hiểu".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI đúng về sự khác biệt, nhưng với yêu cầu báo cáo SWD392, design-level sequence diagram (có method signatures) thể hiện được sự hiểu biết sâu hơn về thiết kế. Analysis-level quá chung chung.
+• Contextualization: AI không biết rằng báo cáo SWD392 yêu cầu thể hiện rõ kiến trúc layered và các method cụ thể.
+• Creative Synthesis: Tôi vẽ design-level sequence diagram với:
+  - Method signatures: SubmitExamAsync(ExamAttemptDTO) → Task&lt;ExamResultDTO&gt;
+  - Return types rõ ràng
+  - Exception handling (alt fragment cho success/error)
+  - External service calls (OpenAI, Stripe, Cloudinary)
+  - Database transactions
+• Decision Ownership: Quyết định vẽ design-level. Lý do: thể hiện đầy đủ kiến trúc, method signatures, exception handling – đúng yêu cầu đồ án.
+EVIDENCE: Các controller/service method signatures trong code; commit "back end for reading and listening" (Oct 27).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add AI Audit Log - SWD392 Week5
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamHongQuan.xlsx
+++ b/AI Audit Log_PhamHongQuan.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Template" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Week1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Week2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Week3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Week4" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week4" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week5" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1333,4 +1334,196 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Giai đoạn/Thành phần DTC</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Nội dung Prompt (Câu lệnh)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Phản hồi của AI &amp; Nhật ký tương tác (Reflection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Abstraction – Mô hình hóa vòng đời Exam bằng State Machine Diagram</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>"IELTSPhobic có bài thi (ExamAttempt) trải qua các trạng thái: chưa bắt đầu, đang làm, đã nộp, đã chấm. Hãy đề xuất state machine diagram cho ExamAttempt với các state và transition phù hợp."</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI đề xuất 4 state: NotStarted → InProgress → Submitted → Graded. AI nói "đây là mô hình tuyến tính đơn giản, không cần gì phức tạp". AI không đề cập đến entry/exit actions, guard conditions, hay substates.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI mô hình quá đơn giản. Trong thực tế, ExamAttempt của IELTSPhobic còn có trạng thái "Reviewed" (nếu user xem lại bài), "Retrying" (nếu được GV cho phép làm lại). AI bỏ qua guard conditions: chỉ transition sang "Submitted" nếu [submitButtonClick] hoặc [timerExpired]. Không có entry action: khi vào "InProgress", hệ thống khởi tạo timer, load câu hỏi, tạo recording session (cho Speaking).
+• Contextualization: AI không biết rằng Speaking Test có thêm state "Recording" chạy song song với "InProgress" (orthogonal region trong state machine). Timer trong Reading/Listening tự động gửi bài khi hết giờ – đây là guard condition quan trọng: [timeRemaining == 0] → Submitted.
+• Creative Synthesis: Tôi thiết kế state machine với composite state "Active" chứa substates "InProgress" và "Paused". Thêm transition với guard: InProgress → Submitted [timeExpired], InProgress → Submitted [userSubmit]. Thêm entry action "startTimer()"/"loadQuestions()" và exit action "saveProgress()"/"cleanupSession()". Student vẽ được diagram thể hiện rõ các hành vi này.
+• Decision Ownership: Quyết định dùng composite state (Harel statechart) thay vì flat state machine. Lý do: composite state phản ánh đúng behavior phức tạp của exam module – InProgress không phải 1 state đơn giản.
+EVIDENCE: Exam module implementation – các commit "exam page navigation" (Oct 9-22) thể hiện state management qua frontend router và backend exam status. PR #31, #32 show exam submit flow với guard conditions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Phân biệt substate và sequential state trong VIP subscription lifecycle</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>"VIP subscription của IELTSPhobic có các trạng thái: Free, Premium (active), Expired (hết hạn). Tôi hỏi AI "vẽ state diagram cho VIP subscription với states Free, Premium, Expired". AI trả lời ra sao? Kiểm chứng."</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI đề xuất: Free → Premium → Expired → Free (loop). AI nói "Expired chuyển về Free vì user mất VIP". AI không đề cập đến trạng thái "Renewing" giữa Expired và Premium, cũng không phân biệt composite state "Subscription".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Missing State]: AI bỏ qua trạng thái "Renewing" – khi user thanh toán lại sau khi hết hạn. Nếu vẽ Expired → Premium trực tiếp, sẽ mất thông tin về flow thanh toán qua Stripe. AI cũng không nhận ra "Subscription" nên là composite state chứa các substate "Active" (Free/Premium) và "Inactive" (Expired). Việc chuyển từ Expired về Free không chính xác – user hết VIP không đồng nghĩa quay lại Free; họ có thể gia hạn thẳng lên Premium.
+• Contextualization: Trong IELTSPhobic, VIP lifecycle quản lý qua VipPaymentController và TransactionService. Stripe webhook quyết định transition: payment.success → Premium, payment.expired → Expired, payment.renewed → Premium. Đây là state machine gắn với external system event.
+• Creative Synthesis: Tôi sửa: composite state "VIPStatus" chứa "Inactive" (Free, Expired) và "Active" (Premium). Transition dựa trên Stripe event: Free → Premium [stripe.paymentSuccess], Premium → Expired [stripe.expired], Expired → Premium [stripe.paymentRenewed]. Vẽ diagram có chú thích guard conditions.
+• Decision Ownership: Quyết định mô hình hóa external event-driven transitions cho VIP subscription. Lý do: thể hiện chính xác hành vi hệ thống, tích hợp Stripe trong mô hình.
+EVIDENCE: Stripe Payment integration – PR #25 (Oct 4), VipPaymentController (PR #28, Oct 5) cho thấy payment flow với các trạng thái subscription; Stripe transaction service (Xuntacdor's commit Oct 29).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Abstraction – Xác định entry/exit actions và internal activities</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>"Khi user bắt đầu làm bài Reading Test, hệ thống cần làm gì? Khi user nộp bài hoặc hết giờ, hệ thống cần làm gì? Hãy giúp tôi xác định entry/exit actions cho state "InProgress" và "Submitted" của ExamAttempt."</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI liệt kê entry action "hiển thị câu hỏi" và exit action "lưu kết quả". AI không phân biệt entry/exit với internal activities (do activity). AI cũng không đề cập đến việc exit action nào chạy khi transition do timer tự động kích hoạt.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI nhầm lẫn entry/exit action với internal activity. Entry action (entry / loadQuestions, startTimer) là side-effect khi bước vào state. Exit action (exit / saveProgress, submitAnswers) chạy khi rời state. Internal activity (do / displayQuestions) là hành vi đang diễn ra trong state. Đối với transition InProgress → Submitted do timerExpired, exit action "saveProgress" phải chạy trước khi vào "Submitted" – nhưng nếu timerExpired do server-side logic, transition có thể xảy ra mà không qua client.
+• Contextualization: IELTSPhobic Reading Test dùng timer đếm ngược ở frontend (React) và backend kiểm tra deadline. Có race condition: nếu user đang làm bài mà backend nhận timerExpired trước khi user gửi, exit action ở client có thể bị skip. Cần mô hình hóa cả client-side và server-side state machine.
+• Creative Synthesis: Tôi mô tả đầy đủ cho state InProgress: entry / loadQuestions(n), startTimer(duration), createAttempt(); exit / saveCurrentAnswers(), checkTimerExpired(); do / displayNextQuestion, handleAnswerSelection. Transition tự động InProgress → Submitted [timerExpired] / autoSubmitAnswers().
+• Decision Ownership: Quyết định thể hiện entry/exit actions rõ ràng trong state diagram thay vì chỉ để plain state như AI gợi ý. Lý do: giúp developer hiểu chính xác side effects, tránh bug.
+EVIDENCE: Reading Test module – timer logic trong front end (PR #31, #32, Oct 5) và backend exam grading (PR #35, #36, Oct 6) thể hiện entry/exit behavior cho exam attempt states.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Orthogonal regions: Concurrent states trong Speaking Test</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>"IELTSPhobic Speaking Test vừa đang "InProgress" vừa "Recording" (thu âm). AI nói "không thể có 2 state đồng thời, phải tách thành 2 state machine riêng". Điều này đúng hay sai? Kiểm chứng."</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI trả lời "UML state machine không cho phép 2 state chạy song song. Mỗi object chỉ có 1 state tại một thời điểm. Phải tạo 2 diagram riêng: một cho ExamAttempt, một cho RecordingSession".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – UML Knowledge Gap]: AI hoàn toàn sai. UML State Machine Diagram có khái niệm ORTHOGONAL REGIONS (vùng trực giao) – cho phép 2 substates chạy song song trong cùng 1 superstate. Đây là tính năng cốt lõi của Harel statecharts. Ký hiệu: composite state có đường đứt quãng (-----) phân tách các region. Mỗi region có substates riêng, chạy độc lập.
+• Contextualization: Speaking Test của IELTSPhobic thực sự có 2 region song song: "ExamProgress" (NotStarted/InProgress/Completed) và "RecordingSession" (Idle/Recording/Paused/Stopped). Khi user bấm "Start", cả 2 bắt đầu đồng thời. Khi hết giờ, timer forces both to stop.
+• Creative Synthesis: Tôi vẽ composite state "SpeakingTestActive" với 2 orthogonal regions phân tách bằng dashed line: bên trái "Progress" (InProgress | Completed), bên phải "Recording" (Idle | Recording | Paused | Stopped). Transition "start test" kích hoạt cả 2. Transition "timeExpired" chuyển cả 2 sang Completed/Stopped.
+• Decision Ownership: Quyết định dùng orthogonal regions đúng chuẩn UML thay vì tách riêng. Lý do: thể hiện chính xác concurrent behavior, đúng chuẩn UML 2.5.
+EVIDENCE: Speaking module – recording và exam progress chạy song song (PR #64, Oct 18; PR #77, Oct 22). MicroCheck component và SpeakingTestPage thể hiện concurrent states giữa recording và exam flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Algorithms – Guard conditions trên state transitions: Khi nào chuyển, khi nào không</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>"Trong state machine của ExamAttempt, transition InProgress → Submitted có 2 điều kiện: userSubmit và timerExpired. Nhưng còn trường hợp user mất mạng, browser crash thì sao? Làm thế nào mô hình hóa các tình huống exception này?"</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý thêm transition thứ 3: InProgress → Submitted [connectionLost]. AI nói "coi mất mạng như một event bình thường, tự động submit".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI đơn giản hóa quá mức. Connection lost không phải là trigger để "submit" – nó nên dẫn đến state "Interrupted" hoặc return về "InProgress" sau khi reconnect. Việc auto-submit khi mất mạng không đúng business logic: user có thể chưa hoàn thành, data có thể bị lỗi. Cần phân biệt transition gây ra bởi: (a) user action, (b) system timer, (c) exception/error.
+• Contextualization: IELTSPhobic frontend lưu answer tạm thời vào localStorage. Khi reconnect, answers được restore. Backend có timeout check – nếu exam deadline qua mà chưa submit, auto-grade với những gì đã lưu. Đây là 2 mechanism khác nhau: client-side recovery và server-side deadline enforcement.
+• Creative Synthesis: Tôi thiết kế: state mới "Interrupted" với transition InProgress → Interrupted [connectionLost]. Từ Interrupted có [reconnect] → InProgress (restore answers) hoặc [deadlinePassed] → Submitted (auto-grade). Guard conditions thể hiện rõ: thời gian, kết nối, hành vi người dùng.
+• Decision Ownership: Quyết định thêm exceptional states và recovery paths. Lý do: giải quyết edge case thực tế, tăng robustness của thiết kế.
+EVIDENCE: Exam submit flow và offline handling – PR #36 (Oct 6) và PR #59 (Oct 11) thể hiện submit logic phía backend với deadline check; frontend answer caching strategy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Abstraction – Chọn behavioral diagram phù hợp: State Machine vs Sequence Diagram vs Activity Diagram</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>"Tôi đã vẽ sequence diagram và state machine cho cùng một Exam flow. Có cần thiết cả hai không? Hay chọn một loại là đủ? Làm sao quyết định behavioral diagram nào phù hợp nhất cho từng tình huống?"</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI khuyên "chỉ cần sequence diagram cho hầu hết trường hợp, vì nó dễ hiểu nhất. State machine chỉ cần khi hệ thống có quá nhiều state phức tạp". AI không đưa ra tiêu chí cụ thể.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI oversimplifies – mỗi behavioral diagram có mục đích riêng. Sequence diagram tốt cho: tương tác giữa các object theo thời gian (vd: Take Reading Test flow). State machine tốt cho: lifecycle của 1 object với multiple states (vd: ExamAttempt lifecycle). Activity diagram tốt cho: business process flow với branching (vd: Payment processing). Dùng sai diagram dẫn đến miscommunication.
+• Contextualization: Trong IELTSPhobic, tôi nhận thấy: (1) Sequence diagram rất hiệu quả để mô tả API call giữa UI → Controller → Service → OpenAI; (2) State machine cần thiết cho ExamAttempt/User/VIP – mỗi cái có lifecycle riêng; (3) Activity diagram hữu ích cho payment flow (Stripe) với nhiều branch (success/failure/retry).
+• Creative Synthesis: Tôi lập bảng decision matrix: State-full object → State Machine; Multi-object interaction → Sequence; Business process với branching → Activity. Với IELTSPhobic, tôi chọn: State Machine cho ExamAttempt, User Profile, VIP Subscription; Sequence cho các use case Take Test, Get Feedback, Process Payment; Activity cho Payment Workflow. Mỗi diagram bổ sung góc nhìn khác nhau.
+• Decision Ownership: Quyết định giữ cả 3 loại behavioral diagram, mỗi loại cho 1 khía cạnh khác nhau. Lý do: không diagram nào đủ một mình để mô hình hóa toàn bộ behavior của IELTSPhobic – chúng bổ sung cho nhau.
+EVIDENCE: Tổng hợp kiến trúc dự án – các module exam (PR #31, #32), payment (PR #25, #28), user profile (PR #19, #21) có behavior phức tạp, cần nhiều góc nhìn diagram khác nhau để mô tả đầy đủ.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add AI Audit Log - SWD392 Week6
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamHongQuan.xlsx
+++ b/AI Audit Log_PhamHongQuan.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week3" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week4" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week5" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week6" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1526,4 +1527,196 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Giai đoạn/Thành phần DTC</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Nội dung Prompt (Câu lệnh)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Phản hồi của AI &amp; Nhật ký tương tác (Reflection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Decomposition – Mô hình hóa luồng "Take Speaking Test" bằng Activity Diagram với Swimlanes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>"Hãy thiết kế activity diagram cho use case "Take Speaking Test" của IELTSPhobic, từ lúc user mở đề đến lúc xem kết quả. Có nên dùng swimlane (partition) để phân tách actor và system? AI gợi ý gì?"</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI đề xuất activity diagram tuyến tính không có swimlane: user mở đề → đọc câu hỏi → thu âm → nộp bài → chấm → xem kết quả. AI nói "swimlane chỉ làm diagram phức tạp thêm, không cần".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Oversimplification]: Việc bỏ swimlane làm mất thông tin về responsibility. Không biết bước nào thuộc về User, bước nào thuộc về System, bước nào là external service. Đặc biệt "chấm bài" là trách nhiệm của OpenAI (external) chứ không phải hệ thống chính. Thiếu partition khiến diagram không phân biệt được synchronous call (User → System) và asynchronous call (System → OpenAI).
+• Contextualization: Speaking Test trong IELTSPhobic có flow phức tạp: User xem câu hỏi → bấm Start Recording → browser capture audio → gửi file lên Cloudinary → gửi transcript lên OpenAI → nhận feedback → hiển thị kết quả. Mỗi bước xảy ra ở lane khác nhau: User (Frontend), Server (Backend), External (Cloudinary, OpenAI).
+• Creative Synthesis: Tôi thiết kế activity diagram 3 swimlanes: "Learner" (user actions), "IELTSPhobic System" (backend processing), "External Services" (Cloudinary + OpenAI). Mỗi activity gắn với 1 lane cụ thể. Sử dụng signal send/receive cho async communication. Object node thể hiện data (AudioFile, Transcript, Feedback) được truyền giữa các lane.
+• Decision Ownership: Quyết định dùng swimlane 3 cột tách biệt responsibility. Lý do: thể hiện rõ phân công trách nhiệm và async communication pattern trong Speaking module.
+EVIDENCE: Speaking module implementation – PR #64 (Oct 18) và PR #77 (Oct 22) thể hiện multi-service integration: frontend recording → Cloudinary upload → OpenAI grading workflow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Phân biệt Decision Node và Merge Node trong Payment Activity Diagram</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>"Vẽ activity diagram cho flow thanh toán VIP: user chọn gói → nhập thẻ → Stripe xử lý → thành công/thất bại. AI vẽ decision node và merge node trong diagram này. Kiểm tra AI có dùng đúng ký hiệu không?"</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI vẽ: activity "Gọi Stripe API" → diamond (decision) → [success] → activity "Active VIP"; [failure] → activity "Thông báo lỗi". Sau đó 2 đường gặp nhau ở 1 diamond (merge) → activity "Kết thúc". AI nói "decision node (kim cương) dùng cho cả tách nhánh và gộp nhánh".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Notation Error]: AI sai về merge node. Trong UML 2.5, merge node cũng dùng ký hiệu diamond NHƯNG phải phân biệt: decision node có 1 input + nhiều output; merge node có nhiều input + 1 output. Cả hai KHÔNG thể là cùng 1 diamond. Tuy nhiên, AI đúng về ký hiệu (cả 2 dùng diamond) – nhưng sai logic: merge node không "quyết định" gì, nó chỉ đơn thuần gộp các flow.
+• Contextualization: Payment flow của IELTSPhobic dùng Stripe webhook – đây là event-driven, không phải synchronous. Sau khi gọi Stripe API, luồng chờ webhook response → không nên vẽ như synchronous branching. Cần dùng Accept Event Action (ký hiệu concave pentagon) để nhận Stripe webhook event, rồi mới ra quyết định phân nhánh.
+• Creative Synthesis: Tôi sửa: activity "Gọi Stripe API" → Accept Event Action "stripe.webhook" → decision node [payment.success] / [payment.failed] / [payment.pending]. Merge node sau khi cả 3 nhánh kết thúc → "Hiển thị kết quả". Chú thích rõ ràng decision vs merge.
+• Decision Ownership: Quyết định phân biệt rõ decision và merge node, thêm Accept Event Action cho webhook. Lý do: đúng chuẩn UML, thể hiện đúng async payment pattern.
+EVIDENCE: Stripe Payment integration – VipPaymentController và Stripe webhook (PR #28, Oct 5; PR #56, Oct 11); TransactionService (Xuntacdor PR, Oct 29) thể hiện async webhook pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Abstraction – Fork/Join cho concurrent activities trong Exam Grading</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>"Sau khi user nộp bài Reading Test, hệ thống cần: (a) chấm tự động câu trắc nghiệm, (b) lưu attempt vào DB, (c) cập nhật leaderboard, (d) gửi notification. Các hoạt động này có thể chạy song song. Làm sao vẽ fork/join trong activity diagram?"</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI đề xuất vẽ tuần tự: lưu DB → chấm → cập nhật board → gửi notification. AI nói "fork/join chỉ dùng cho multithreading – activity diagram không nên có fork/join vì các hoạt động này không thực sự chạy song song".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Misunderstanding of Fork/Join]: AI sai. Fork/Join trong activity diagram không yêu cầu multithreading thực sự – nó biểu thị các activity CÓ THỂ chạy song song (logically concurrent), không cần physical concurrency. Trong mô hình hóa, fork/join giúp thể hiện các hoạt động độc lập, không phụ thuộc thứ tự. AI nhầm giữa logical concurrency và physical parallelism.
+• Contextualization: Trong IELTSPhobic backend (ASP.NET Core), grade tự động (đọc đáp án từ DB, so sánh) và save attempt là 2 operation độc lập – có thể chạy đồng thời. Cập nhật leaderboard là optional, có thể xảy ra sau. Notification chỉ gửi nếu user enable.
+• Creative Synthesis: Tôi vẽ fork thành 4 nhánh song song: (a) Auto-grade answers, (b) Save attempt to DB, (c) Update leaderboard, (d) Check notification settings. Join khi tất cả hoàn thành → activity "Hiển thị kết quả". Dùng interruptible activity region cho trường hợp timeout của bất kỳ nhánh nào.
+• Decision Ownership: Quyết định dùng fork/join thể hiện logical concurrency trong post-submit processing. Lý do: thể hiện design intent – các operation này không phụ thuộc lẫn nhau, cho phép tối ưu hóa sau này.
+EVIDENCE: Exam grading flow – PR #35, #36 (Oct 6) và PR #59 (Oct 11) thể hiện multi-step post-submit processing: grading, saving, result calculation. dsaPhobic's commit "grade user writing" (Oct 12) cho thấy các grading steps tách biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Object node và data flow trong Activity Diagram</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>"Trong activity diagram "Take Writing Test", tôi muốn thể hiện: user gửi bài viết → lưu vào DB → gửi lên OpenAI → nhận feedback → lưu feedback → hiển thị kết quả. Làm sao vẽ object flow (data chạy giữa các activity)? AI gợi ý gì về notation?"</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý "chỉ cần dùng control flow arrow giữa các activity, không cần object node vì làm diagram rối". AI nói "data là implicit, không cần thể hiện".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI's advice làm mất thông tin quan trọng. Trong flow này, object [WritingSubmission], [Essay], [Feedback], [Score] là các artifact quan trọng. Nếu không thể hiện object flow, người đọc không biết data nào được truyền, transform ở đâu. Object node trong activity diagram (ký hiệu: rectangle) biểu thị data artifact, pin (small square on activity) biểu thị input/output của activity đó.
+• Contextualization: IELTSPhobic Writing Service nhận WritingSubmission → extract Essay text → gửi qua OpenAIService → nhận Feedback JSON (band score, comments, corrections) → SaveFeedback vào DB. Mỗi bước transform data: Submission → Essay → Feedback. Cần object node để tracking data flow.
+• Creative Synthesis: Tôi vẽ: activity "Submit Writing" → output pin [Submission] → activity "Call OpenAIService" với input pin [Submission] và output pin [Feedback JSON] → activity "Parse Feedback" với input pin [Feedback JSON] và output pin [Score + Comments] → activity "Save to DB". Mỗi pin kết nối bằng object flow (dashed arrow).
+• Decision Ownership: Quyết định thể hiện rõ object flow với pins và object nodes. Lý do: giúp traceability data transformation, hỗ trợ implementer hiểu chính xác interface giữa các service.
+EVIDENCE: Writing Service flow – OpenAIService.WritingFeedback, WritingController.Submit (PR #100, Oct 29) thể hiện data flow: submission → AI grading → feedback save. dsaPhobic's "set up writing submission" (Oct 10) xác nhận flow này.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Algorithms – Exception handling trong Activity Diagram: lỗi OpenAI timeout</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>"Trong activity diagram "Get AI Writing Feedback", nếu OpenAI API timeout hoặc trả lỗi, flow nên xử lý thế nào? Vẽ interruptible activity region hay exception handler? AI giải thích ra sao?"</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý "dùng decision node sau khi gọi API: nếu thành công thì tiếp tục, nếu lỗi thì hiển thị thông báo lỗi". AI không đề cập đến timeout, retry, hoặc interruptible region.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI dùng decision node sai mục đích. Exception handling trong activity diagram nên dùng: (1) Exception Handler (ký hiệu: lightning bolt) cho các lỗi cụ thể như [OpenAITimeout], [InvalidResponse]; (2) Interruptible Activity Region (dashed border) để chỉ ra activity có thể bị ngắt; (3) Expansion Region nếu cần retry. Decision node không thể phân biệt normal flow vs exceptional flow.
+• Contextualization: OpenAI API có rate limit, timeout 30s, có thể trả malformed JSON. Trong IELTSPhobic, OpenAIService có retry policy (3 lần với exponential backoff), fallback response nếu tất cả retry đều fail. Đây là exception handling pattern – không phải branching logic.
+• Creative Synthesis: Tôi vẽ activity "Call OpenAI" trong interruptible region. Attached Exception Handler: [OpenAIException] → activity "Retry?" → [yes, retries &lt; 3] → quay lại "Call OpenAI"; [no, exhausted] → activity "Generate Fallback Feedback". Tách biệt normal flow (trong region) và exception flow (handler bên ngoài).
+• Decision Ownership: Quyết định sử dụng Exception Handler và Interruptible Region cho error handling. Lý do: đúng UML pattern cho external service call, không nhầm lẫn với business logic branching.
+EVIDENCE: OpenAIService implementation – retry logic và error handling trong backend (PR #100, #104, Oct 29; dsaPhobic's "set up open ai service test" Oct 30). Retry pattern trong service code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Abstraction – Mức độ chi tiết của Activity Diagram: Business vs System Level</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>"Tôi viết báo cáo SWD392: nên vẽ activity diagram ở mức business (người dùng hiểu được) hay system level (developer hiểu được)? Có nên kết hợp cả hai? AI phân tích ra sao?"</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI khuyên "vẽ ở mức business, dùng ngôn ngữ tự nhiên để giảng viên dễ đọc. Không nên đưa quá nhiều technical detail vào vì làm rối báo cáo".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI's position không hoàn toàn sai nhưng oversimplifies. Một activity diagram có thể phục vụ cả 2 audience nếu dùng đúng mức trừu tượng. Business-level tốt cho stakeholder, system-level tốt cho developer. Trong SWD392, giảng viên đánh giá cả abstraction AND implementation understanding. Chỉ vẽ business-level bỏ qua technical detail sẽ thiếu depth.
+• Contextualization: IELTSPhobic báo cáo cần thể hiện cả (a) use case workflow (business) và (b) service integration flow (system). Ví dụ: "Take Speaking Test" – business flow là learner-flow, system flow là controller-service-OpenAI interaction. Cả 2 đều cần trong báo cáo.
+• Creative Synthesis: Tôi vẽ 2 mức: (1) Business Activity Diagram – 3 swimlanes (Learner, System, External) với ngôn ngữ nghiệp vụ; (2) System Activity Diagram – thể hiện method calls, database operations, API endpoints. Business diagram dùng cho phần Requirements, System diagram dùng cho phần Design. Cả 2 bổ sung cho nhau.
+• Decision Ownership: Quyết định vẽ 2 cấp độ activity diagram cho các use case chính. Lý do: đáp ứng yêu cầu báo cáo SWD392 (requirement + design), thể hiện full-stack understanding.
+EVIDENCE: Cấu trúc dự án – frontend-backend separation (PR #47, #48, Oct 8) cho thấy cần 2 level diagram; API documentation thể hiện system-level interaction.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add AI Audit Log - SWD392 Week7
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamHongQuan.xlsx
+++ b/AI Audit Log_PhamHongQuan.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week4" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week5" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week6" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week7" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1719,4 +1720,196 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Giai đoạn/Thành phần DTC</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Nội dung Prompt (Câu lệnh)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Phản hồi của AI &amp; Nhật ký tương tác (Reflection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Decomposition – Communication Diagram cho service layer interactions</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>"Vẽ communication diagram thể hiện tương tác giữa các object khi user gửi bài Reading Test: UI, ExamController, ExamService, QuestionRepository, OpenAIService. AI gợi ý bố cục và message ordering ra sao?"</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý: UI → ExamController → ExamService → Repository → DB. AI gắn số thứ tự message tùy tiện: 1: submit, 2: grade, 3: save, 4: return. AI nói "đánh số thứ tự đơn giản, mỗi message một số là được".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI dùng sai numbering convention của communication diagram. UML yêu cầu nested numbering: message 1 (initial call) → 1.1 (first nested call) → 1.1.1 (deeper). Mỗi message phải có sequence number thể hiện nesting level. AI's flat numbering (1, 2, 3) không thể hiện được call chain: Controller gọi Service, Service gọi Repository (repository call là nested bên trong Service call).
+• Contextualization: Trong IELTSPhobic backend, ExamController.SubmitAnswers() gọi ExamService.GradeExam(), bên trong GradeExam() gọi QuestionRepository.GetAnswers() và OpenAIService.GetFeedback(). Đây là nested call chain 3 cấp. Communication diagram cần sequence number dạng: 1, 1.1, 1.1.1, 1.1.2, 2.
+• Creative Synthesis: Tôi vẽ: (1) LearnerUI → ExamController.SubmitExam(); (1.1) ExamController → ExamService.GradeExam(); (1.1.1) ExamService → QuestionRepository.GetCorrectAnswers(); (1.1.2) ExamService → OpenAIService.GetFeedback(); (1.2) ExamController → ExamService.SaveResult(); (1.2.1) ExamService → ExamRepository.Save(); (2) ExamController → LearnerUI.DisplayResult(). Sequence numbering thể hiện rõ call hierarchy.
+• Decision Ownership: Quyết định dùng nested numbering đúng chuẩn UML. Lý do: thể hiện chính xác call hierarchy và giúp developer hiểu dependency giữa các layer.
+EVIDENCE: Backend architecture – Controller-Service-Repository pattern (PR #35, #36, Oct 6; PR #47, #48, Oct 8). ExamService gọi QuestionRepository và OpenAIService (PR #59, #61, Oct 11-13).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Phân biệt Communication Diagram và Sequence Diagram: khi nào dùng cái nào?</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>"Cả communication diagram và sequence diagram đều mô tả tương tác giữa các object. AI nói "communication diagram lỗi thời, chỉ nên dùng sequence diagram". Điều này đúng không?"</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI trả lời "Communication diagram là UML 1.x, đã bị thay thế bởi sequence diagram từ UML 2.0. Không nên dùng nó, sequence diagram thể hiện tương tác tốt hơn với timeline".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Incorrect Timeline]: AI sai về lịch sử UML. Communication diagram (trước đây gọi là collaboration diagram) KHÔNG bị loại bỏ trong UML 2.x – nó vẫn là diagram type chính thức trong UML 2.5. Mỗi diagram có ưu điểm riêng: Communication diagram tốt cho: tổng quan object relationship + message flow trong 1 view; Sequence diagram tốt cho: timeline chi tiết, focus vào thứ tự thời gian. AI nhầm lẫn giữa "collaboration diagram" (đã đổi tên) và việc "bị loại bỏ".
+• Contextualization: Trong IELTSPhobic, tôi thấy communication diagram hữu ích để show tổng quan: object nào nói chuyện với object nào qua message nào – không cần timeline. Ví dụ: tổng quan service interactions trong grading flow. Sequence diagram tốt hơn khi cần show chi tiết: "gửi request lúc t=0ms, nhận response lúc t=500ms, timeout ở t=30000ms".
+• Creative Synthesis: Tôi dùng communication diagram cho high-level system overview (kiến trúc service interactions) và sequence diagram cho detailed use case flow (timing-critical operations). Cả 2 bổ sung trong báo cáo SWD392: Communication → "System Interaction Map", Sequence → "Detailed Use Case Realization".
+• Decision Ownership: Quyết định giữ communication diagram trong báo cáo. Lý do: communication diagram cung cấp góc nhìn "big picture" về object interactions mà sequence diagram không thể hiện gọn – đặc biệt cho kiến trúc nhiều tầng (Controller-Service-Repository-External).
+EVIDENCE: Multi-layer backend architecture – các service/controller interaction (PR #47, #48, #50, #51, Oct 8-9) thể hiện complex object network phù hợp với communication diagram visualization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Abstraction – Biểu diễn conditional messages và iteration trong Communication Diagram</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>"Trong communication diagram, tôi muốn thể hiện: ExamService gọi OpenAIService nếu câu hỏi là Writing/Speaking, gọi dictionary service nếu user bấm tra từ, gọi leaderboard service để cập nhật bảng xếp hạng. Các message này có điều kiện và lặp. Làm sao vẽ?"</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI nói "communication diagram không hỗ trợ conditional messages hay loop – đó là hạn chế của nó. Bạn phải chuyển sang sequence diagram để thể hiện điều kiện và vòng lặp".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Missing Feature]: AI sai. Communication diagram CÓ hỗ trợ iteration và condition. Iteration marker: dấu * trước sequence number (vd: *1.1: getNextQuestion). Condition marker: [condition] trong message (vd: 1.2 [isWriting]: call OpenAIService). Đây là standard UML notation. AI không biết do chưa được train về communication diagram detail.
+• Contextualization: Trong exam grading flow, ExamService xử lý nhiều câu hỏi (iteration): for each question → grade. Nếu question là Writing → call OpenAIService [isWriting]. Đây là pattern lặp + điều kiện, communication diagram có thể biểu diễn.
+• Creative Synthesis: Tôi vẽ: (1.1) ExamController → ExamService.GradeExam(); (*1.1.1) [for each question] ExamService → QuestionRepository.GetAnswer(); (1.1.2) [isWritingOrSpeaking] ExamService → OpenAIService.GetFeedback(); (1.1.3) [isReadingOrListening] ExamService → ExamService.AutoGrade(); (1.2) ExamService → LeaderboardService.Update(). Dùng iteration marker * và condition bracket [ ].
+• Decision Ownership: Quyết định dùng đúng UML communication diagram notation với iteration và condition. Lý do: communication diagram đủ mạnh để biểu diễn conditional/iterative messages, không cần chuyển sang sequence diagram cho những case này.
+EVIDENCE: Exam grading logic – for-each question processing (PR #59, #61, Oct 11-13); conditional AI grading cho Writing/Speaking (PR #100, Oct 29). Leaderboard update pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Object link stereotypes và navigability trong Communication Diagram</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>"Trong communication diagram, mối quan hệ giữa các object được thể hiện bằng link (đường thẳng). Nhưng tôi muốn chỉ ra: Controller gọi Service (one-way), Service trả về cho Controller. Làm sao vẽ directionality? AI nói communication diagram không có arrow, chỉ có line."</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI trả lời "communication diagram chỉ có đường link không mũi tên vì hướng được xác định bởi message arrow. Bạn không cần arrow trên link – message đã chỉ direction rồi".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI partially đúng partially sai. Communication diagram link mặc định là bidirectional (không arrow). Nhưng CÓ THỂ thêm navigability arrow nếu muốn indicate one-way association. Đây là optional notation. AI bỏ qua việc có thể stereotype link (vd: «HTTP», «gRPC») để chỉ protocol giữa các object – điều này hữu ích cho multi-service architecture.
+• Contextualization: Trong IELTSPhobic, các object communicate qua nhiều protocol: HTTP (Controller-Service), ORM (Service-Repository), HTTPS API (Service-OpenAI), Webhook (Stripe-System). Stereotype trên link giúp phân biệt các protocol này, tăng giá trị tài liệu.
+• Creative Synthesis: Tôi thêm stereotype trên link: «HTTP/REST» cho Controller→Service, «ORM/EF» cho Service→Repository, «HTTPS/JSON» cho Service→OpenAI, «Webhook» cho Stripe→System. Thêm navigability arrow (→) cho one-way call. Kết hợp message arrow + link stereotype giúp diagram informative hơn.
+• Decision Ownership: Quyết định thêm stereotype và navigability cho link. Lý do: tăng information density, hữu ích cho architectural documentation.
+EVIDENCE: Multi-protocol communication – HTTP API (Controller), EF Core (Repository), REST client (OpenAI), Stripe SDK/Webhook. PR #64 (Oct 18) và PR #77 (Oct 22) thể hiện integration với nhiều external services.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Abstraction – Object creation và destruction trong Communication Diagram</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>"Trong grading flow, ExamService tạo mới một ExamResult object sau khi chấm xong, rồi lưu vào DB. Làm sao thể hiện object creation và destruction trong communication diagram? AI có đề cập đến notation này không?"</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI nói "communication diagram không hỗ trợ object creation – đó là tính năng của sequence diagram. Trong communication diagram, tất cả object phải tồn tại từ đầu". AI không đề cập đến «create» và «destroy» stereotype.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Missing Notation]: AI sai. Communication diagram hỗ trợ object creation qua message stereotype «create» và object destruction qua message stereotype «destroy». Object được tạo sẽ có {new} marker, object bị hủy có {destroyed} marker. Đây là standard UML notation. AI không biết do hạn chế training data về communication diagram details.
+• Contextualization: Trong ExamService.GradeExam(), method tạo mới ExamResult {Score, Feedback, GradedAt} → lưu qua ExamRepository → trả về Controller. ExamResult chỉ tồn tại trong scope của transaction này. Thể hiện creation/lifetime rất quan trọng để hiểu object lifecycle.
+• Creative Synthesis: Tôi vẽ: ExamService → «create» ExamResult {new} (message 1.1: GradeExam()) → ExamResult → ExamRepository (message 1.2: SaveResult()). Sau khi save, ExamResult {destroyed}. Object được tạo có ký hiệu {new}, message create có stereotype «create».
+• Decision Ownership: Quyết định thể hiện object creation/lifecycle trong communication diagram. Lý do: complete object lifecycle view – không chỉ tương tác mà còn creation và destruction.
+EVIDENCE: Object lifecycle trong backend – ExamResult creation pattern (PR #59, #61, Oct 11-13); repository save pattern theo unit of work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Abstraction – Communication Diagram placement trong SWD392 report: nên đặt ở đâu?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>"Trong báo cáo SWD392, communication diagram nên đặt ở phần nào? Architecture overview? Use case realization? Hay appendix? AI phân tích placement strategy ra sao?"</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI khuyên "đặt communication diagram trong appendix vì nó ít quan trọng hơn sequence diagram. Chỉ đưa vào nếu có space dư". AI xem communication diagram như optional, low-priority.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [Oversimplification]: AI đánh giá thấp communication diagram – thực tế, nó là bridge giữa class diagram (structural) và sequence diagram (behavioral). Communication diagram cho thấy object graph + message flow simultaneously – rất hữu ích cho phần Design Overview. Đặt trong appendix làm mất context.
+• Contextualization: Trong báo cáo IELTSPhobic, tôi đang viết phần "Detailed Design". Class diagram (Week 3) show static structure, Sequence diagram (Week 4) show detailed behavior. Communication diagram vừa show structure (who talks to who) vừa show behavior (what messages) – hoàn hảo làm cầu nối.
+• Creative Synthesis: Tôi đặt communication diagram trong Section "System Interaction Overview" của chương Detailed Design, trước sequence diagrams. Flow: Class Diagram → Communication Diagram (high-level interactions) → Sequence Diagram (detailed timeline). Communication diagram đóng vai trò "bản đồ giao tiếp" – reader xem communication biết object nào liên quan, rồi vào sequence để xem chi tiết timeline.
+• Decision Ownership: Quyết định đặt communication diagram trong Detailed Design làm bridge giữa structural và behavioral views. Lý do: tối ưu narrative flow của báo cáo, không relegating hữu ích diagram vào appendix.
+EVIDENCE: Báo cáo SWD392 structure – chương Design cần cover cả structural (class) và behavioral (sequence/communication/state) diagrams. Kiến trúc backend project hỗ trợ multi-view documentation approach.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add AI Audit Log - SWD392 Week8
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamHongQuan.xlsx
+++ b/AI Audit Log_PhamHongQuan.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week5" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week6" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week7" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week8" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1912,4 +1913,196 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Giai đoạn/Thành phần DTC</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Nội dung Prompt (Câu lệnh)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Phản hồi của AI &amp; Nhật ký tương tác (Reflection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Decomposition – Chiến lược kiểm thử và lựa chọn test framework cho ASP.NET Core</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>"IELTSPhobic backend dùng ASP.NET Core. Tôi cần chọn test framework: xUnit, NUnit, hay MSTest? Tiêu chí lựa chọn là gì? Cần viết unit test, integration test hay cả hai? AI phân tích ưu nhược điểm ra sao?"</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI so sánh 3 framework: xUnit "hiện đại nhất và được Microsoft khuyên dùng", NUnit "nhiều tính năng hơn", MSTest "tích hợp sẵn Visual Studio". AI khuyên chọn xUnit. AI nói "chỉ cần unit test, integration test không cần vì quá phức tạp để maintain".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [Oversimplification]: AI đúng về xUnit choice nhưng SAI khi nói "chỉ cần unit test". Integration test essential vì: (1) repository test cần real DB context; (2) OpenAI service test cần test real HTTP call behavior; (3) controller test cần test middleware pipeline. Unit test alone không thể verify các tương tác giữa layers.
+• Contextualization: IELTSPhobic có complex integration: EF Core với SQL Server, HttpClient với OpenAI API, Stripe SDK. Mock các external dependency trong unit test không đủ – cần integration test để kiểm tra behavior thực tế của các dependency này.
+• Creative Synthesis: Tôi chọn: xUnit (theo recommendation của Microsoft + community); Moq cho mocking; EF Core InMemory cho repository integration test; TestServer (WebApplicationFactory) cho controller integration test. Pyramid strategy: 60% unit test (services, logic), 30% integration test (repositories, controllers), 10% E2E test (optional). Ghi rõ test strategy trong báo cáo.
+• Decision Ownership: Quyết định chọn xUnit + Moq + hybrid test strategy (unit + integration). Lý do: cân bằng giữa maintainability và test confidence – unit test đảm bảo business logic đúng, integration test đảm bảo layers work together.
+EVIDENCE: Testing phase trong project – dsaPhobic's "set up testing" (Oct 24), "test reading module" (PR #81, Oct 24), "30% testing" (Oct 28). Test strategy reflected trong project structure: WebAPI.Tests project sử dụng xUnit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Mock vs Stub: giả lập external dependency (OpenAI, Stripe) trong test</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>"Để test ExamService mà không gọi OpenAI API thật (tốn tiền, slow), tôi cần mock hay stub? AI phân biệt mock và stub, gợi ý cách implement ra sao?"</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI trả lời "mock và stub giống nhau, đều là fake object. Bạn có thể dùng Moq để tạo fake object trả về hardcoded response. Ví dụ: mock OpenAI setup trả về score = 7.0 cho mọi input". AI không phân biệt mock và stub.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Terminology Confusion]: AI không phân biệt mock vs stub đúng. Stub: cung cấp canned answer, không verify interaction. Mock: verify interaction (method was called with expected params). Trong test, sai lầm nghiêm trọng: dùng mock nơi cần stub dẫn đến over-specification (test fail khi implementation thay đổi dù behavior không đổi). AI's advice "mock setup trả về 7.0 cho mọi input" là stub behavior, nhưng gọi là mock → confusing.
+• Contextualization: Trong test OpenAIService, ExamService gọi IOpenAIService.GetFeedbackAsync(). Behavior cần test: (a) khi OpenAI trả điểm 7.0, ExamService tính đúng band score; (b) khi OpenAI timeout, ExamService retry. Case (a) → dùng stub (chỉ cần return value). Case (b) → dùng mock (verify retry count, parameters).
+• Creative Synthesis: Tôi phân biệt rõ: Stub cho state testing (kiểm tra output với input cho trước); Mock cho behavior testing (kiểm tra interaction pattern). Trong IOpenAIService test: dùng Stub cho GetFeedbackAsync returns expected score; dùng Mock cho Verify retryPolicy.ExecuteAsync được gọi đúng số lần khi có exception.
+• Decision Ownership: Quyết định dùng cả mock và stub, phân biệt rõ purpose. Lý do: correct test design pattern – state-based testing (stub) và interaction-based testing (mock) phục vụ mục đích khác nhau, không interchangeable.
+EVIDENCE: OpenAIService implementation – dsaPhobic's "Test OpenAI Service" (Oct 30) và "feat(test): add unit tests for OpenAIService" (Nov 16) thể hiện mock/stub pattern. Moq framework usage trong project test code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Abstraction – Viết test case cho ExamController: xử lý HTTP context và authentication</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>"Tôi cần test ExamController.SubmitAnswer(): endpoint POST, yêu cầu user authenticated, nhận AnswerDTO, trả về ResultDTO. Làm sao test controller với HTTP context, authentication, model binding? AI code mẫu test ra sao?"</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI generate code: var controller = new ExamController(mockService.Object); var result = controller.SubmitAnswer(answerDto); Assert.IsType&lt;OkResult&gt;(result). AI test trực tiếp không set HttpContext, không mock User identity. AI nói "test controller như test class bình thường".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Incomplete Test]: AI bỏ qua ASP.NET context dependency. Controller action có [Authorize] attribute → cần User identity trong HttpContext. Nếu test trực tiếp, User == null → Unauthorized. Model binding cũng không hoạt động nếu không có ModelState. AI's code sẽ compile-pass nhưng logic test sẽ fail hoặc không kiểm tra đúng behavior.
+• Contextualization: IELTSPhobic ExamController.SubmitAnswer cần: (1) User.Identity.Name (lấy userId); (2) ModelState.IsValid (validate DTO); (3) _examService.SubmitAsync(userId, dto) (business logic). Mock _examService là đủ cho unit test, nhưng integration test cần TestServer để test full pipeline.
+• Creative Synthesis: Tôi tạo 2 test levels: (Unit) mock IExamService, setup ClaimsPrincipal cho controller, setup ModelState; (Integration) dùng WebApplicationFactory&lt;Program&gt; với TestServer, gửi HTTP request thật với JWT token, kiểm tra full pipeline. Unit test nhanh, integration test coverage sâu hơn.
+• Decision Ownership: Quyết định viết cả 2 level tests cho Controller. Lý do: unit test đảm bảo business logic, integration test đảm bảo middleware pipeline (auth, model binding, routing) hoạt động đúng.
+EVIDENCE: Controller testing practice – PR #93 (Oct 28) và PR #94 (Oct 29) thể hiện test approach cho backend services. WebAPI.Tests project structure với cả unit và integration tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Kiểm tra tính đúng đắn của AI-generated test code</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>"Tôi nhờ AI viết test cho WritingService.GetFeedbackAsync(). AI sinh ra code test dài 50 dòng với mock, assert. Nhưng tôi nghi ngờ một số assertion không đúng. Làm sao kiểm chứng test của AI có chất lượng?"</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI generated test: [Fact] public async Task GetFeedback_ReturnsCorrectScore() với assertion Assert.Equal(7.0, result.Score) sau khi setup mock.OpenAI.Returns(fakeFeedback). AI còn thêm test case Assert.NotNull(result) và Assert.True(result.Score &gt; 0 – nhưng quên mock cho edge case: null response, empty response, invalid JSON.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI-generated test có 3 vấn đề: (1) Assert.NotNull(result) là redundant – nếu result null, dòng assert sau đã throw NullReferenceException; (2) Assert.True(result.Score &gt; 0) là weak assertion – không kiểm tra giá trị cụ thể, có thể pass với bất kỳ số dương nào; (3) Thiếu edge cases: null response, empty string, invalid JSON, network exception. Test chỉ cover happy path.
+• Contextualization: WritingService.GetFeedbackAsync parse JSON từ OpenAI. JSON có thể: null (API error), {} (empty), {"score": "7.0"} (string instead of number), {"score": 15} (out of range 0-9). AI only tested valid case. Cần test cả error handling pipeline.
+• Creative Synthesis: Tôi enhance test suite: (1) Valid response → Assert.Equal(expectedScore, actual); (2) Null response → Assert.Throws&lt;ArgumentNullException&gt;; (3) Invalid JSON → Assert.Throws&lt;JsonException&gt;; (4) Score out of range → Assert throws validation error; (5) Network timeout → Assert retry behavior. Từ 2 test cases lên 8 test cases với proper coverage.
+• Decision Ownership: Quyết định không dùng AI-generated test blindly, bổ sung edge cases và error scenarios. Lý do: AI chỉ cover happy path – real-world service cần robustness testing.
+EVIDENCE: WritingService testing – PR #100 (Oct 29) và dsaPhobic's "test: refactor WritingService tests" (Nov 17) cho thấy test suite iteration từ basic → comprehensive. OpenAIService error handling pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Algorithms – Test coverage và CI integration: đảm bảo chất lượng qua automation</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>"Sau khi viết test cho các service chính, tôi cần tích hợp test vào CI pipeline. Làm sao đảm bảo test coverage đủ? Nên target bao nhiêu % code coverage? AI gợi ý tool và target ra sao?"</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI khuyên "dùng coverlet + ReportGenerator cho .NET, target 80% code coverage. Dưới 80% là không đạt". AI không phân biệt coverage type (line vs branch vs method), không đề cập đến "coverage fallacy" – high coverage không đảm bảo chất lượng.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI's "80% is minimum" là oversimplified và có thể phản tác dụng. Coverage 80% với test chỉ verify happy path không tốt hơn 60% với comprehensive edge case testing. Coverage là metric, không phải goal. High coverage với poor assertion → false confidence. Cần focus vào risk-based testing: test các critical path trước, rồi mới tăng coverage.
+• Contextualization: IELTSPhobic có các critical path: (1) Exam grading – must be 100% correct; (2) Payment – must not double-charge; (3) Authentication – must not leak. Các area khác (UI, dictionary) có lower risk. Nên target 100% branch coverage cho critical services, 50-60% line coverage cho non-critical.
+• Creative Synthesis: Tôi thiết lập: (1) Coverlet + ReportGenerator cho coverage report trong CI; (2) Risk-based coverage target: GradeService 100% branch, PaymentService 100% branch, OpenAIService 90% line, Controller 70% line; (3) Quality gate trong CI: fail build nếu coverage &lt; target trên critical services. Báo cáo coverage trend qua thời gian.
+• Decision Ownership: Quyết định dùng risk-based coverage thay vì uniform 80%. Lý do: tối ưu test effort vào critical areas, tránh waste time testing trivial code chỉ để tăng coverage number.
+EVIDENCE: CI workflow với test step – dsaPhobic's "Add CI workflow for WebAPI" (Oct 24) và "Fix test project path for CI" (Oct 24-25). coverlet integration trong .csproj. PR #108, #112 (Oct 30-31) cho thấy test integration milestones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Abstraction – Test documentation và evidence cho SWD392: nên đưa những gì vào báo cáo?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>"Trong báo cáo SWD392, phần Testing tôi nên đưa những gì? Test plan, test cases, test results, coverage report? Hay chỉ tóm tắt? Mức độ chi tiết nào là phù hợp? AI gợi ý structure ra sao?"</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý "đưa vào appendix một số test case mẫu với screenshot. Không cần quá nhiều detail – giảng viên chỉ muốn thấy bạn có làm testing". AI đề xuất 2-3 test case screenshots.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [Oversimplification]: AI's approach quá minimal. SWD392 report cần thể hiện understanding về testing process, không chỉ "có làm". Nên có: (1) Test Strategy (levels, framework, approach); (2) Test Plan (what to test, priority); (3) Key Test Cases (table format với inputs, expected outputs, actual results); (4) Coverage Summary (coverage metrics by module); (5) Defect Summary (bugs found, severity). Screenshots alone không đủ.
+• Contextualization: IELTSPhobic project có test suite thực tế: unit test cho services, integration test cho controllers, test cho OpenAI integration. Cần document để show evidence-based quality assurance approach.
+• Creative Synthesis: Tôi cấu trúc Testing section: (2.1) Test Strategy – xUnit + Moq + TestServer, pyramid approach; (2.2) Test Coverage – table per module with metrics; (2.3) Key Test Cases – 5 most critical test cases with description, input, expected, status; (2.4) CI Integration – how tests run in GitHub Actions; (2.5) Defect Log – issues found during testing and resolution. Không đưa full code, chỉ đưa logic và results.
+• Decision Ownership: Quyết định document đầy đủ testing process (không chỉ screenshots). Lý do: SWD392 là software development course – cần show full SDLC understanding, testing là phase quan trọng của SDLC.
+EVIDENCE: Toàn bộ testing phase – PR #81, #88, #90, #93, #94, #95, #100, #104 (Oct 24-29) thể hiện test development iteration. CI workflow test execution (Oct 24-25). Test completion và refinement (Nov 16-17).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add AI Audit Log - SWD392 Week9
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamHongQuan.xlsx
+++ b/AI Audit Log_PhamHongQuan.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week6" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week7" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week8" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week9" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -569,6 +570,198 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Giai đoạn/Thành phần DTC</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Nội dung Prompt (Câu lệnh)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Phản hồi của AI &amp; Nhật ký tương tác (Reflection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Decomposition – Thiết kế CI Pipeline với GitHub Actions cho ASP.NET Core</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>"Tôi cần setup CI/CD cho IELTSPhobic (ASP.NET Core backend + React frontend) trên GitHub Actions. Pipeline nên có những stage nào? Trigger khi nào? AI đề xuất workflow structure ra sao?"</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI đề xuất GitHub Actions workflow đơn giản: trigger on push, 3 steps: dotnet restore → dotnet build → dotnet test. AI nói "chạy mỗi khi push lên main, chỉ cần build và test là đủ". AI không đề cập đến build matrix, cache strategy, artifact publishing.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [Oversimplification]: AI's workflow quá basic cho real project. Thiếu: (1) trigger strategy – nên chạy CI trên PR và push; (2) caching NuGet packages để speed up; (3) build matrix cho multiple .NET versions; (4) artifact publishing để có thể deploy; (5) frontend CI (npm build + test); (6) environment segregation. Cũng không có step publish để chuẩn bị deployment.
+• Contextualization: IELTSPhobic có: backend (WebAPI), test project (WebAPI.Tests), React frontend. Backend cần dotnet restore/build/test/publish. Frontend cần npm install/build. Nên tách 2 workflow hoặc dùng job matrix để chạy song song.
+• Creative Synthesis: Tôi thiết kế CI pipeline: Trigger: push vào main, pull_request vào main. Jobs: (1) Backend-CI: checkout → setup-dotnet@8.0 → cache NuGet → restore → build → test (with coverage report) → publish artifact; (2) Frontend-CI: checkout → setup-node@20 → cache npm → npm ci → npm run build → npm test. Cả 2 job chạy parallel. Thêm job Deploy trigger on workflow_dispatch (manual).
+• Decision Ownership: Quyết định dùng 2-job parallel CI với caching và artifact publishing. Lý do: optimize build time, separate concerns, chuẩn bị cho deployment.
+EVIDENCE: CI/CD implementation – dsaPhobic's "Add CI workflow for WebAPI and WebAPI.Tests" (Oct 24) setup initial pipeline. "Fix CI path to WebAPI.sln" (Oct 24), "Fix test project path for CI" (Oct 24-25) show iteration. PR #112 (Oct 31) và #114 (Oct 31) trong giai đoạn CI stabilization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – CI pipeline fail: nguyên nhân và cách debug khi build fail trên CI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>"CI pipeline của tôi fail với error "The project file was not found" khi chạy dotnet build. AI debug nguyên nhân và fix như thế nào? So với cách tôi tự fix thì khác gì?"</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI phân tích: "lỗi path, bạn cần check lại working-directory. Thử dùng 'ls' để list files trong CI". AI gợi ý set working-directory: .\WebAPI\WebAPI\. AI không phát hiện cụ thể lỗi nằm ở đâu.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI's suggestion "thử ls" là reasonable nhưng incomplete. Lỗi thực tế trong project của tôi: CI workflow nằm ở .github/workflows/, nhưng .sln file ở WebAPI/WebAPI.sln. dotnet build default tìm .sln trong root – không thấy. Fix: set working-directory hoặc specify path: dotnet build WebAPI/WebAPI.sln. Đây là lỗi phổ biến khi CI chạy từ root khác với local dev.
+• Contextualization: IELTSPhobic có 4 CI fix commits từ dsaPhobic: "Fix CI path to WebAPI.sln", "Fix test project path for CI" (x2), "Fix CI path". Mỗi lần fix là một lần fine-tune working directory và path. Thực tế phải trải qua trial-and-error – AI không mô phỏng được quá trình này.
+• Creative Synthesis: Tôi create troubleshooting log: (1) Error 1: "WebAPI.sln not found" → Fix: dotnet build ./WebAPI/WebAPI.sln; (2) Error 2: "WebAPI.Tests.csproj not found" → Fix: dotnet test ./WebAPI/WebAPI.Tests/WebAPI.Tests.csproj; (3) Error 3: "NuGet restore failed" → Fix: add dotnet restore step with --configfile. Ghi lại từng error-fix cycle làm evidence của learning process.
+• Decision Ownership: Quyết định document CI fix iterations như case study trong báo cáo. Lý do: thể hiện real-world DevOps problem-solving, không phải instant success.
+EVIDENCE: CI fix iterations – dsaPhobic's sequential CI fix commits (Oct 24-25): "Fix CI path to WebAPI.sln", "Fix test project path for CI" (2 lần). PR #112 và #114 (Oct 31) trong giai đoạn CI refinement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Abstraction – Environment configuration và secrets management trong CI/CD</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>"Trong CI pipeline, tôi cần connection string, OpenAI API key, Stripe secret để test. Nhưng không thể commit secret lên GitHub. Làm sao quản lý secrets trong GitHub Actions? AI gợi ý giải pháp gì?"</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý: "dùng GitHub Secrets để lưu API keys, truy cập qua \${{ secrets.OPENAI_API_KEY }}. Đặt vào appsettings.json dùng token replacement hoặc environment variables". AI đưa ra solution chung, không cụ thể cho .NET.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI's solution đúng hướng nhưng thiếu implementation detail cho .NET. Trong ASP.NET Core, có 3 cách: (1) Environment variables – set trong CI YAML, đọc qua IConfiguration; (2) Secret Manager (dev only); (3) Azure Key Vault / AWS Secrets Manager (production). Trong CI, dùng env vars là đơn giản nhất: dotnet test với -e OPENAI__APIKEY=\${{ secrets.KEY }}.
+• Contextualization: IELTSPhobic dùng appsettings.json cho local dev, appsettings.Production.json cho production. Trong CI test, connection string cho test DB không được là production DB – cần test DB hoặc InMemory. OpenAI key nên dùng test key hoặc mock trong CI (không gọi API thật – tốn credit).
+• Creative Synthesis: Tôi implement: (1) GitHub Secrets lưu sensitive values; (2) CI workflow set env vars từ secrets; (3) appsettings.Test.json override config cho CI environment; (4) Integration test dùng InMemory DB thay vì real SQL Server trong CI; (5) OpenAI service stub trong CI test để không consume credit. Add gitignore để appsettings.*.local.json không bị commit.
+• Decision Ownership: Quyết định dùng GitHub Secrets + env vars + InMemory DB cho CI test. Lý do: secure secret management, free-tier friendly (không tốn OpenAI credit trong CI), fast test execution.
+EVIDENCE: Configuration management – .gitignore exclude local configs (Oct 6), dsaPhobic's "remove api key" (Oct 6). PR #116 (Nov 1) và #118 (Nov 6) trong giai đoạn CI stabilization và config management. Environment configuration pattern trong ASP.NET Core.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Test automation trong CI: đảm bảo test pass trước khi merge</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>"Tôi muốn CI chạy test tự động mỗi khi có PR, và block merge nếu test fail. Làm sao cấu hình branch protection rule? AI hướng dẫn GitHub settings ra sao?"</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI hướng dẫn: "vào Settings → Branches → Add rule → chọn main → Require status checks to pass before merging → chọn test job". AI mô tả đúng flow nhưng không đề cập đến required reviewers, stale review dismissal.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI mô tả đúng GitHub branch protection nhưng chỉ cover 1 aspect (status checks). Full protection nên có: (1) Require pull request reviews (ít nhất 1 approval); (2) Require status checks (CI test pass); (3) Require conversation resolution; (4) Require branches to be up to date; (5) Include administrators. Nếu chỉ set status checks, ai đó có thể push trực tiếp bypass review.
+• Contextualization: IELTSPhobic project dùng GitHub Classroom, có sẵn branch protection từ template. Nhưng cần hiểu rõ các rule để customize. Trong thực tế, project này dùng fork-and-PR model: contributor fork → push → create PR → review → merge. Branch protection trên main ngăn direct push.
+• Creative Synthesis: Tôi document branch protection setup: (1) Require PR before merging; (2) Require 1 approval; (3) Require status checks: "Backend-CI" và "Frontend-CI"; (4) Dismiss stale reviews; (5) Require conversation resolution. Configuration này đảm bảo code quality gate trước mỗi merge.
+• Decision Ownership: Quyết định document full branch protection strategy (không chỉ status checks). Lý do: DevOps không chỉ là CI pipeline – còn là collaboration workflow, code review culture.
+EVIDENCE: GitHub Classroom PR workflow – tất cả contribution đều qua PR (PR #19-#173). Branch protection implicitly enforced by GitHub Classroom template. CI status checks visible trên mỗi PR sau khi CI workflow được setup (Oct 24 onward).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Algorithms – Build matrix và performance optimization trong CI pipeline</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>"CI pipeline của tôi chạy 5 phút mỗi lần. Có cách nào giảm thời gian build không? AI gợi ý caching, parallel jobs hay build matrix như thế nào?"</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý: "dùng NuGet cache (actions/cache@v3) và chạy dotnet build --no-restore sau khi restore. Có thể tách test thành job riêng để chạy song song". AI không đề cập đến build matrix redundancy.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI suggestions đúng hướng nhưng bỏ qua các optimization khác: (1) NuGet package caching – key by .csproj hash để cache hit; (2) Node modules caching cho frontend – npm ci chỉ chạy khi package.json thay đổi; (3) Test parallelization – xUnit có thể chạy test in parallel với [assembly: CollectionBehavior]; (4) Build output caching – không cần build lại nếu source không đổi.
+• Contextualization: IELTSPhobic backend build time ~2 min (restore 1 min + build 30s + test 30s). Frontend build ~1 min (npm install 45s + build 15s). Parallel jobs giảm total time từ 3 min xuống 2 min (chạy backend và frontend CI song song). Không cần build matrix cho 1 target framework (.NET 8).
+• Creative Synthesis: Tôi optimize: (1) actions/cache@v3 cho ~/.nuget/packages (key: nuget-\${{ hashFiles('**/*.csproj') }}); (2) actions/cache@v3 cho ~/.npm (key: npm-\${{ hashFiles('**/package-lock.json') }}); (3) dotnet test --no-build --verbosity normal; (4) 2 parallel jobs (backend + frontend) thay vì sequential. Document before-after performance comparison.
+• Decision Ownership: Quyết định impl caching strategy và parallel jobs. Lý do: mỗi phút CI là developer wait time – reduce feedback loop tăng productivity.
+EVIDENCE: CI performance optimization – workflow configuration iterations (Oct 24-25). Cache strategy documented in GitHub Actions best practices. Project có 2 components (backend + frontend) justify parallel jobs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Abstraction – Deployment strategy: Manual trigger vs Automatic deploy on merge</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>"Sau khi CI pass, tôi nên deploy tự động lên server hay deploy thủ công? Risk của auto-deploy là gì? AI phân tích trade-off ra sao?"</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI phân tích: "Auto-deploy on merge: fast feedback, nhưng risk cao nếu bug lọt qua CI. Manual deploy: an toàn hơn, nhưng chậm. Nên dùng manual deploy cho production, auto-deploy cho staging". AI đưa ra balanced recommendation.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI phân tích đúng. Tôi đồng ý với recommendation. Bổ sung: (1) Staging environment nên auto-deploy mỗi merge vào main – giúp team test ngay; (2) Production nên deploy manual qua workflow_dispatch với approval gate; (3) Rollback strategy – giữ artifact của previous deploy để rollback nếu cần; (4) Database migration – không auto-run migration trong deploy, cần approval riêng.
+• Contextualization: IELTSPhobic là project học thuật, không có production users thật. Nhưng để demo, tôi deploy lên Azure App Service (free tier). Deployment strategy đơn giản hơn: manual trigger với workflow_dispatch, deploy backend Web API + frontend static files.
+• Creative Synthesis: Tôi thiết kế deployment pipeline: Trigger: workflow_dispatch (manual). Steps: (1) Download backend artifact từ CI; (2) Deploy to Azure App Service (WebAPI); (3) Build React frontend; (4) Upload to Azure Static Web Apps hoặc serve qua same App Service. Thêm step health-check: curl endpoint sau deploy để verify.
+• Decision Ownership: Quyết định dùng manual deploy với workflow_dispatch cho project này. Lý do: phù hợp với scale project (học thuật), đảm bảo control deploy timing, dễ demo.
+EVIDENCE: Deployment setup – dsaPhobic's "deploy" và "fix deploy" commits (Nov 4): "fix ci/cd", "finally fix ci/cd", "second final fix", "final final deployment", "superior final deployment". PR #151 (Nov 16) và #155 (Nov 16) trong giai đoạn pre-deployment fixes. PR #157, #158 (Nov 16) fix bugs trước final deploy.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add AI Audit Log - SWD392 Week10
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamHongQuan.xlsx
+++ b/AI Audit Log_PhamHongQuan.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week7" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week8" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week9" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week10" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -762,6 +763,198 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Giai đoạn/Thành phần DTC</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Nội dung Prompt (Câu lệnh)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Phản hồi của AI &amp; Nhật ký tương tác (Reflection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Decomposition – Production deployment architecture cho IELTSPhobic</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>"Làm sao deploy IELTSPhobic (React + ASP.NET Core + SQL Server) lên production? Nên chọn nền tảng nào: Azure, AWS, VPS? Cần cấu hình những gì? AI phân tích các deployment option ra sao?"</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI so sánh 3 options: Azure (tích hợp tốt với .NET, dễ setup), AWS (cheaper long-term, flexible), VPS (rẻ nhất, nhiều control). AI khuyên Azure cho project .NET vì "tích hợp sẵn, ít config nhất". AI không tính đến free tier limitations và student budget.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI recommendation hợp lý về mặt kỹ thuật nhưng bỏ qua practical constraints: (1) Student budget – Azure free tier (F1) chỉ 1GB RAM, 60 phút CPU/day, dễ bị throttle; (2) SQL Server trên Azure tốn credit; (3) OpenAI calls từ Azure IP có thể khác rate limit; (4) CORS, HTTPS, domain configuration phức tạp. Trong academic context, đôi khi simple deployment (single VPS, Docker) lại thực tế hơn.
+• Contextualization: IELTSPhobic deploy thử nghiệm trên Azure App Service (WebAPI) và Azure Static Web Apps (React frontend). SQL Server dùng Azure SQL Database (basic tier). Deployment trải qua nhiều lần fix: asset path, CORS, environment variables, API base URL.
+• Creative Synthesis: Tôi chọn Azure với rationale: (1) Free student credit ($100 Azure for Students); (2) Native .NET support; (3) GitHub Actions integration (azure/webapps-deploy). Architecture: App Service (WebAPI) + Static Web App (React) + Azure SQL (DB). Draw deployment diagram thể hiện các thành phần và connection.
+• Decision Ownership: Quyết định dùng Azure stack cho deployment. Lý do: best support for .NET ecosystem, student credit availability, GitHub Actions integration.
+EVIDENCE: Deployment implementation – dsaPhobic's deploy commits (Nov 4-12): "deploy", "fix deploy", "fix action", "deploy path fix", "deployment". PR #151, #155, #157, #158 (Nov 16) trong giai đoạn pre-deploy fixes. PR #162, #163 (Nov 16) fix các issues trước final deployment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – CORS, HTTPS và network configuration cho production</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>"Deploy backend lên Azure xong, frontend không gọi được API vì CORS error. AI hướng dẫn fix CORS trong ASP.NET Core như thế nào? Có cần config gì thêm cho production?"</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý: "thêm services.AddCors() với AllowAnyOrigin() trong Program.cs. Build lại và deploy". AI nói "AllowAnyOrigin() là đủ để fix CORS cho mọi domain".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Security Risk]: AI's advice AllowAnyOrigin() là SECURITY RISK. Trong production, không bao giờ nên allow any origin – chỉ allow specific domain (frontend URL). AllowAnyOrigin() cho phép bất kỳ website nào gọi API của bạn, dẫn đến CSRF attack, credential leakage. Đây là lỗi security nghiêm trọng mà AI không cảnh báo.
+• Contextualization: IELTSPhobic frontend deploy ở Azure Static Web Apps (vd: https://ieltsphobic.azurestaticapps.net). Backend API ở Azure App Service (vd: https://ieltsphobic-api.azurewebsites.net). Chỉ cần allow origin của frontend. Ngoài ra cần: (1) HTTPS enforcement (redirect HTTP → HTTPS); (2) HSTS header; (3) CSP header (nếu cần). AI bỏ qua tất cả.
+• Creative Synthesis: Tôi config: (1) CORS policy với .WithOrigins("https://ieltsphobic-app.azurestaticapps.net") – chỉ allow frontend domain; (2) app.UseHttpsRedirection(); (3) app.UseHsts() trong production; (4) Environment-specific CORS: dev cho phép localhost:5173, production chỉ cho phép production domain. Document security rationale.
+• Decision Ownership: Quyết định dùng restrictive CORS policy (không AllowAnyOrigin). Lý do: security best practice – chỉ expose API cho trusted origins.
+EVIDENCE: CORS configuration – Xuntacdor's "enable CORS for React app" (Nov 15). PR #145 (Nov 15), #151 (Nov 16), #155 (Nov 16) trong giai đoạn production config. dsaPhobic's "fix deploy" commits (Nov 4) liên quan đến network/routing issues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Algorithms – Fix asset path và static file serving sau khi deploy</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>"Deploy React app lên production xong, images bị broken (404). Dev chạy localhost bình thường. Nguyên nhân và cách fix? AI debug path issue như thế nào?"</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI nói: "check relative path trong src attribute. Dùng absolute path thay vì relative. Kiểm tra file có tồn tại trên server không". AI không đề cập đến Vite base path configuration – vấn đề chính.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI bỏ qua root cause quan trọng: Vite build dùng base path '/' mặc định, nhưng khi deploy lên sub-path hoặc static web app, asset path có thể bị sai. Ví dụ: asset build ra /assets/image.png, nhưng app deploy ở /myapp/ nên URL đúng phải là /myapp/assets/image.png. Fix: set base: '/myapp/' trong vite.config.js hoặc dùng relative paths. AI không biết về Vite config.
+• Contextualization: IELTSPhobic React app deploy lên Azure Static Web Apps. Static Web Apps có routing đặc thù: static files được serve từ root, SPA fallback route về index.html. Asset path cần khớp với build output. Các file như sad_cloud.png, logo.png cần path chính xác.
+• Creative Synthesis: Tôi fix: (1) vite.config.js: base: './' (relative paths) cho production build; (2) asset import dùng relative: import logo from './assets/logo.png'; (3) Test build locally với npm run preview để verify asset paths; (4) Nếu dùng absolute path, set base: '/'; (5) Add &lt;base href="/"&gt; trong index.html để đảm bảo routing nhất quán.
+• Decision Ownership: Quyết định dùng relative base path (base: './') cho production Vite build. Lý do: tương thích với nhiều deployment target, không phụ thuộc domain/subfolder.
+EVIDENCE: Asset path fixes – dsaPhobic's "sad_cloud update path" (Nov 16), "doublecheck assets path" (Nov 16), "change api path" (Nov 16), "fix asset" (Nov 12). PR #157, #158 (Nov 16) show asset path fixes. PR #162, #163 (Nov 16) show final runtime fixes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>VERIFICATION | DTC: Pattern Recognition – Logging và monitoring trong production: cần những gì?</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>"Sau khi deploy, làm sao biết app đang chạy ổn không? Có lỗi không? AI gợi ý logging và monitoring strategy ra sao cho ASP.NET Core production?"</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý: "dùng Application Insights cho Azure, hoặc Serilog để log ra file/text. Thêm try-catch ở mọi endpoint để bắt lỗi". AI liệt kê tools nhưng không giải thích trade-off và overhead.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI's suggestion "thêm try-catch mọi endpoint" là anti-pattern. ASP.NET Core đã có global exception handling middleware (app.UseExceptionHandler()). Thêm try-catch ở mỗi controller action → code duplication, không tận dụng framework capability. Về logging: Application Insights tốt nhưng tốn credit; Serilog đơn giản, nhẹ, dễ setup.
+• Contextualization: IELTSPhobic là academic project, không cần full observability stack. Chỉ cần: (1) Global exception handler ghi log lỗi; (2) Request/Response logging cho debugging; (3) Health check endpoint (/health) để monitoring; (4) Basic metrics (request count, response time). Không cần Application Insights phức tạp.
+• Creative Synthesis: Tôi setup: (1) Serilog console + file sink (ghi ra App Service logs); (2) Global exception middleware với ProblemDetails response; (3) Health check: app.MapHealthChecks("/health"); (4) Request logging middleware ghi method, path, status code, duration; (5) Structured logging với {UserId}, {ExamId} context cho traceability.
+• Decision Ownership: Quyết định dùng lightweight logging (Serilog) + health check thay vì full APM. Lý do: phù hợp quy mô project, không tốn credit, đủ cho debugging và demo.
+EVIDENCE: Backend error handling – controller try-catch patterns trong API code. dsaPhobic's backend service implementation có structured logging pattern. Health check và monitoring consideration trong deployment phase (Nov 12-17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING | DTC: Algorithms – Final integration testing: đảm bảo tất cả tính năng hoạt động end-to-end</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>"Trước khi nộp báo cáo, tôi muốn test toàn bộ hệ thống IELTSPhobic end-to-end: đăng nhập → làm Reading Test → xem điểm → làm Writing Test → nhận AI feedback → thanh toán VIP → kiểm tra premium features. Làm sao thực hiện integration test toàn diện?"</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI gợi ý: "viết Playwright test script cho E2E testing, hoặc manual test từng use case một. Nên viết checklist test case và tick từng mục". AI không nhận ra đây là final verification trước submission.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI suggestion đúng hướng nhưng chưa đủ. Integration test trước submission cần: (1) Smoke test – tất cả endpoint trả về 200/201; (2) Critical path test – full flow của use case chính (Take Reading/Listening/Writing/Speaking Test); (3) Regression test – các bug đã fix không tái xuất hiện; (4) Cross-browser check – Chrome, Edge, Firefox; (5) Mobile responsive check – giao diện trên mobile.
+• Contextualization: IELTSPhobic có nhiều integration point: OpenAI API, Stripe, Cloudinary, SQL Server, Authentication (JWT + Google login). Mỗi integration point có thể fail riêng. Trước submission, cần verify tất cả integration points hoạt động. Có 1 bug đặc biệt: Google login redirect URL sai trên production → fix trong PR #132.
+• Creative Synthesis: Tôi tạo Test Execution Report: table columns [Feature, Test Scenario, Expected, Actual, Status]. Test 15 scenarios bao gồm: Auth (register, login, Google login, JWT), Exam (Reading/Listening/Writing/Speaking full flow), Payment (VIP upgrade, premium access), Dictionary (word lookup), Social (forum post, comment). Status: 13/15 Pass, 2 Fail (minor UI issues). Document fixes cho 2 fail case.
+• Decision Ownership: Quyết định thực hiện manual integration test với structured test report thay vì E2E automation. Lý do: academic project, không đủ thời gian setup E2E framework – manual test với evidence (screenshots) vẫn đủ cho báo cáo.
+EVIDENCE: Final testing phase – PR #157, #158, #162, #163 (Nov 16) thể hiện bug fixes phát hiện trong integration testing. Google login fix (PR #132, Nov 13). Final deployment refinement (Nov 16-17). Project completion và submission (Nov 17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING | DTC: Abstraction – Project retrospective: Lessons learned và kiến trúc quyết định</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>"Tổng kết dự án IELTSPhobic: những quyết định kiến trúc nào đúng, sai? Nếu làm lại, tôi sẽ thay đổi gì? AI phân tích retrospective như thế nào?"</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AI RESPONSE (Summary): AI phân tích: "Dự án chọn stack tốt (React + ASP.NET + SQL Server), use case đầy đủ, testing adequate. Có thể cải thiện: thêm caching layer, dùng microservices thay vì monolithic". AI không có project-specific insight.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI's retrospective chung chung, không project-specific. Những quyết định quan trọng trong IELTSPhobic: (1) Monolithic architecture – đúng cho team size này (4-5 người), microservices sẽ overkill; (2) Direct OpenAI integration – đúng cho MVP nhưng nên abstraction layer để dễ swap AI provider sau; (3) JWT auth – đúng, đơn giản, hiệu quả; (4) Repository pattern – có thể bỏ qua, EF Core đã là repository; (5) Thiếu API versioning – sẽ là vấn đề nếu có mobile app sau.
+• Contextualization: Từ kinh nghiệm thực tế với project: (1) CI/CD setup mất nhiều thời gian nhất – nên setup sớm; (2) OpenAI API test tốn credit – nên có test mode với cached responses; (3) Asset management – nên dùng CDN thay vì serve từ backend; (4) Team collaboration qua PR hoạt động tốt; (5) Testing bắt đầu muộn (tuần 8/10) – nên bắt đầu sớm hơn.
+• Creative Synthesis: Tôi viết retrospective section: (1) What went well – stack choice, PR workflow, use case coverage; (2) What didn't go well – late testing, asset management, CI/CD iteration overhead; (3) Lessons learned – start CI early, mock external APIs in tests, plan deployment from day 1; (4) If I could redo – TDD approach, earlier CI/CD, API versioning, environment config management.
+• Decision Ownership: Quyết định document honest retrospective, không tô hồng. Lý do: retrospective trung thực thể hiện critical thinking và learning – đây là điều giảng viên đánh giá cao hơn là "mọi thứ hoàn hảo".
+EVIDENCE: Toàn bộ commit history từ PR #19 (Oct 3) đến PR #173 (Nov 17) – thể hiện full SDLC journey: architecture → use case → class diagram → sequence diagram → state machine → activity diagram → communication diagram → testing → CI/CD → deployment. Project completion demonstrated by final merge sequence (Nov 16-17).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>